<commit_message>
backup: v8 2026-06-07 13:42 IST
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="234">
   <si>
     <t>Timestamp</t>
   </si>
@@ -524,148 +524,145 @@
     <t>PENDING_APPROVAL</t>
   </si>
   <si>
+    <t>APPROVED</t>
+  </si>
+  <si>
+    <t>TKT-00003</t>
+  </si>
+  <si>
+    <t>TKT-00004</t>
+  </si>
+  <si>
+    <t>TKT-00006</t>
+  </si>
+  <si>
+    <t>TKT-00007</t>
+  </si>
+  <si>
+    <t>TKT-00008</t>
+  </si>
+  <si>
+    <t>TKT-00009</t>
+  </si>
+  <si>
+    <t>TKT-00010</t>
+  </si>
+  <si>
+    <t>TKT-00011</t>
+  </si>
+  <si>
+    <t>TKT-00012</t>
+  </si>
+  <si>
+    <t>TKT-00013</t>
+  </si>
+  <si>
+    <t>TKT-00014</t>
+  </si>
+  <si>
+    <t>TKT-00015</t>
+  </si>
+  <si>
+    <t>TKT-00016</t>
+  </si>
+  <si>
+    <t>TKT-00017</t>
+  </si>
+  <si>
+    <t>TKT-00018</t>
+  </si>
+  <si>
+    <t>TKT-00019</t>
+  </si>
+  <si>
+    <t>TKT-00020</t>
+  </si>
+  <si>
+    <t>TKT-00021</t>
+  </si>
+  <si>
+    <t>TKT-00022</t>
+  </si>
+  <si>
+    <t>TKT-00023</t>
+  </si>
+  <si>
+    <t>TKT-00024</t>
+  </si>
+  <si>
+    <t>TKT-00025</t>
+  </si>
+  <si>
+    <t>TKT-00026</t>
+  </si>
+  <si>
+    <t>TKT-00027</t>
+  </si>
+  <si>
+    <t>TKT-00028</t>
+  </si>
+  <si>
+    <t>TKT-00029</t>
+  </si>
+  <si>
+    <t>TKT-00030</t>
+  </si>
+  <si>
+    <t>TKT-00005</t>
+  </si>
+  <si>
+    <t>Ticket ID</t>
+  </si>
+  <si>
+    <t>Date Reported</t>
+  </si>
+  <si>
+    <t>Found at Tower</t>
+  </si>
+  <si>
+    <t>Flat No</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Subcategory</t>
+  </si>
+  <si>
+    <t>Exact Location</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Photo Link</t>
+  </si>
+  <si>
+    <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Date Assigned</t>
+  </si>
+  <si>
+    <t>Target Closure</t>
+  </si>
+  <si>
+    <t>Closure Date</t>
+  </si>
+  <si>
+    <t>Resident Confirmation</t>
+  </si>
+  <si>
+    <t>Reopened</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
     <t>TKT-00002</t>
-  </si>
-  <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
-    <t>TKT-00004</t>
-  </si>
-  <si>
-    <t>TKT-00005</t>
-  </si>
-  <si>
-    <t>TKT-00006</t>
-  </si>
-  <si>
-    <t>TKT-00007</t>
-  </si>
-  <si>
-    <t>TKT-00008</t>
-  </si>
-  <si>
-    <t>TKT-00009</t>
-  </si>
-  <si>
-    <t>TKT-00010</t>
-  </si>
-  <si>
-    <t>TKT-00011</t>
-  </si>
-  <si>
-    <t>TKT-00012</t>
-  </si>
-  <si>
-    <t>TKT-00013</t>
-  </si>
-  <si>
-    <t>TKT-00014</t>
-  </si>
-  <si>
-    <t>TKT-00015</t>
-  </si>
-  <si>
-    <t>TKT-00016</t>
-  </si>
-  <si>
-    <t>TKT-00017</t>
-  </si>
-  <si>
-    <t>TKT-00018</t>
-  </si>
-  <si>
-    <t>TKT-00019</t>
-  </si>
-  <si>
-    <t>TKT-00020</t>
-  </si>
-  <si>
-    <t>TKT-00021</t>
-  </si>
-  <si>
-    <t>TKT-00022</t>
-  </si>
-  <si>
-    <t>TKT-00023</t>
-  </si>
-  <si>
-    <t>TKT-00024</t>
-  </si>
-  <si>
-    <t>TKT-00025</t>
-  </si>
-  <si>
-    <t>TKT-00026</t>
-  </si>
-  <si>
-    <t>TKT-00027</t>
-  </si>
-  <si>
-    <t>TKT-00028</t>
-  </si>
-  <si>
-    <t>TKT-00029</t>
-  </si>
-  <si>
-    <t>TKT-00030</t>
-  </si>
-  <si>
-    <t>TKT-00031</t>
-  </si>
-  <si>
-    <t>Ticket ID</t>
-  </si>
-  <si>
-    <t>Date Reported</t>
-  </si>
-  <si>
-    <t>Found at Tower</t>
-  </si>
-  <si>
-    <t>Flat No</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Subcategory</t>
-  </si>
-  <si>
-    <t>Exact Location</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Photo Link</t>
-  </si>
-  <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Date Assigned</t>
-  </si>
-  <si>
-    <t>Target Closure</t>
-  </si>
-  <si>
-    <t>Closure Date</t>
-  </si>
-  <si>
-    <t>Resident Confirmation</t>
-  </si>
-  <si>
-    <t>Reopened</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>TKT-00003</t>
   </si>
   <si>
     <t>ASSIGNED</t>
@@ -2310,6 +2307,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="13.29"/>
     <col customWidth="1" min="10" max="10" width="29.14"/>
   </cols>
   <sheetData>
@@ -2350,7 +2348,7 @@
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -2386,12 +2384,12 @@
         <v>165</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B3" s="13">
         <v>46152.25501662037</v>
@@ -2423,7 +2421,7 @@
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B4" s="13">
         <v>46152.41155247686</v>
@@ -2458,7 +2456,7 @@
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B5" s="13">
         <v>46152.427458715276</v>
@@ -2493,7 +2491,7 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B6" s="13">
         <v>46152.458851250005</v>
@@ -2528,7 +2526,7 @@
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B7" s="13">
         <v>46167.02062795139</v>
@@ -2560,7 +2558,7 @@
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B8" s="13">
         <v>46172.89509825232</v>
@@ -2590,7 +2588,7 @@
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B9" s="13">
         <v>46174.335368125</v>
@@ -2622,7 +2620,7 @@
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B10" s="13">
         <v>46174.36407401621</v>
@@ -2654,7 +2652,7 @@
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B11" s="13">
         <v>46174.368129826384</v>
@@ -2686,7 +2684,7 @@
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B12" s="13">
         <v>46174.47108636574</v>
@@ -2718,7 +2716,7 @@
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B13" s="13">
         <v>46175.23439052083</v>
@@ -2753,7 +2751,7 @@
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B14" s="13">
         <v>46175.36433582176</v>
@@ -2788,7 +2786,7 @@
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B15" s="13">
         <v>46175.36539417824</v>
@@ -2823,7 +2821,7 @@
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B16" s="13">
         <v>46176.81027090277</v>
@@ -2858,7 +2856,7 @@
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B17" s="13">
         <v>46176.897516701385</v>
@@ -2893,7 +2891,7 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B18" s="13">
         <v>46176.89797092593</v>
@@ -2925,7 +2923,7 @@
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B19" s="13">
         <v>46176.9001487037</v>
@@ -2960,7 +2958,7 @@
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B20" s="13">
         <v>46176.98599523148</v>
@@ -2992,7 +2990,7 @@
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B21" s="13">
         <v>46177.15724104167</v>
@@ -3024,7 +3022,7 @@
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B22" s="13">
         <v>46177.92069255787</v>
@@ -3056,7 +3054,7 @@
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B23" s="13">
         <v>46177.94379626158</v>
@@ -3091,7 +3089,7 @@
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" s="13">
         <v>46177.95516053241</v>
@@ -3126,7 +3124,7 @@
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B25" s="13">
         <v>46178.09025260417</v>
@@ -3158,7 +3156,7 @@
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="13">
         <v>46179.0225042824</v>
@@ -3190,7 +3188,7 @@
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B27" s="13">
         <v>46180.02262467593</v>
@@ -3222,7 +3220,7 @@
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B28" s="13">
         <v>46180.0250299537</v>
@@ -3254,7 +3252,7 @@
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B29" s="13">
         <v>46180.03628767361</v>
@@ -3286,7 +3284,7 @@
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B30" s="13">
         <v>46152.4115727662</v>
@@ -3359,69 +3357,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>199</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>200</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G1" s="16" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="K1" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="L1" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="M1" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="N1" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="P1" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="Q1" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="R1" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="S1" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="T1" s="16" t="s">
         <v>212</v>
-      </c>
-      <c r="T1" s="16" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3450,7 +3448,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3460,7 +3458,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -11585,7 +11583,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C1" s="16" t="s">
         <v>5</v>
@@ -11594,7 +11592,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2">
@@ -11605,13 +11603,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3">
@@ -11628,7 +11626,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4">
@@ -11636,7 +11634,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>13</v>
@@ -11645,12 +11643,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>54</v>
@@ -11662,7 +11660,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6">
@@ -11694,25 +11692,25 @@
         <v>16</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>224</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13">
@@ -11722,17 +11720,17 @@
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17">
@@ -11742,12 +11740,12 @@
     </row>
     <row r="18">
       <c r="B18" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20">
@@ -11762,7 +11760,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -11772,7 +11770,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="18" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v9 2026-06-07 13:43 IST
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="233">
   <si>
     <t>Timestamp</t>
   </si>
@@ -524,15 +524,15 @@
     <t>PENDING_APPROVAL</t>
   </si>
   <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
     <t>TKT-00003</t>
   </si>
   <si>
     <t>TKT-00004</t>
   </si>
   <si>
+    <t>TKT-00005</t>
+  </si>
+  <si>
     <t>TKT-00006</t>
   </si>
   <si>
@@ -606,9 +606,6 @@
   </si>
   <si>
     <t>TKT-00030</t>
-  </si>
-  <si>
-    <t>TKT-00005</t>
   </si>
   <si>
     <t>Ticket ID</t>
@@ -2348,10 +2345,10 @@
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B2" s="13">
-        <v>46151.16717461805</v>
+        <v>46180.05029387731</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>9</v>
@@ -2360,10 +2357,10 @@
         <v>10</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G2" s="10" t="s">
         <v>13</v>
@@ -2372,19 +2369,13 @@
         <v>14</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="L2" s="14">
-        <v>46173.25955616898</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>165</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="K2" s="10"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="10"/>
       <c r="Q2" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3">
@@ -2392,7 +2383,7 @@
         <v>168</v>
       </c>
       <c r="B3" s="13">
-        <v>46152.25501662037</v>
+        <v>46180.05031049768</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>9</v>
@@ -2412,9 +2403,7 @@
       <c r="J3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K3" s="10"/>
       <c r="Q3" s="10" t="s">
         <v>166</v>
       </c>
@@ -2424,7 +2413,7 @@
         <v>169</v>
       </c>
       <c r="B4" s="13">
-        <v>46152.41155247686</v>
+        <v>46180.050328125</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>9</v>
@@ -2447,9 +2436,7 @@
       <c r="J4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K4" s="10"/>
       <c r="Q4" s="10" t="s">
         <v>166</v>
       </c>
@@ -2459,7 +2446,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="13">
-        <v>46152.427458715276</v>
+        <v>46180.05034636574</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>9</v>
@@ -2482,9 +2469,7 @@
       <c r="J5" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K5" s="10"/>
       <c r="Q5" s="10" t="s">
         <v>166</v>
       </c>
@@ -2494,7 +2479,7 @@
         <v>171</v>
       </c>
       <c r="B6" s="13">
-        <v>46152.458851250005</v>
+        <v>46180.0503632176</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>30</v>
@@ -2517,9 +2502,7 @@
       <c r="J6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K6" s="10"/>
       <c r="Q6" s="10" t="s">
         <v>166</v>
       </c>
@@ -2529,7 +2512,7 @@
         <v>172</v>
       </c>
       <c r="B7" s="13">
-        <v>46167.02062795139</v>
+        <v>46180.05037993056</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>9</v>
@@ -2549,9 +2532,7 @@
       <c r="J7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K7" s="10"/>
       <c r="Q7" s="10" t="s">
         <v>166</v>
       </c>
@@ -2561,7 +2542,7 @@
         <v>173</v>
       </c>
       <c r="B8" s="13">
-        <v>46172.89509825232</v>
+        <v>46180.050404814814</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>9</v>
@@ -2579,9 +2560,7 @@
       <c r="J8" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="K8" s="10"/>
       <c r="Q8" s="10" t="s">
         <v>166</v>
       </c>
@@ -2591,7 +2570,7 @@
         <v>174</v>
       </c>
       <c r="B9" s="13">
-        <v>46174.335368125</v>
+        <v>46180.05042226852</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>41</v>
@@ -2605,9 +2584,7 @@
       <c r="F9" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G9" s="10"/>
       <c r="H9" s="10" t="s">
         <v>44</v>
       </c>
@@ -2623,7 +2600,7 @@
         <v>175</v>
       </c>
       <c r="B10" s="13">
-        <v>46174.36407401621</v>
+        <v>46180.05044378473</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>46</v>
@@ -2637,9 +2614,7 @@
       <c r="F10" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G10" s="10"/>
       <c r="H10" s="10" t="s">
         <v>44</v>
       </c>
@@ -2655,7 +2630,7 @@
         <v>176</v>
       </c>
       <c r="B11" s="13">
-        <v>46174.368129826384</v>
+        <v>46180.05046524305</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>50</v>
@@ -2669,9 +2644,7 @@
       <c r="F11" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G11" s="10"/>
       <c r="H11" s="10" t="s">
         <v>44</v>
       </c>
@@ -2687,7 +2660,7 @@
         <v>177</v>
       </c>
       <c r="B12" s="13">
-        <v>46174.47108636574</v>
+        <v>46180.050481909726</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>30</v>
@@ -2701,9 +2674,7 @@
       <c r="F12" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G12" s="10"/>
       <c r="H12" s="10" t="s">
         <v>34</v>
       </c>
@@ -2719,7 +2690,7 @@
         <v>178</v>
       </c>
       <c r="B13" s="13">
-        <v>46175.23439052083</v>
+        <v>46180.05049804398</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>56</v>
@@ -2733,9 +2704,7 @@
       <c r="F13" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G13" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
         <v>14</v>
       </c>
@@ -2754,7 +2723,7 @@
         <v>179</v>
       </c>
       <c r="B14" s="13">
-        <v>46175.36433582176</v>
+        <v>46180.05051513889</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>61</v>
@@ -2768,9 +2737,7 @@
       <c r="F14" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G14" s="10"/>
       <c r="H14" s="10" t="s">
         <v>16</v>
       </c>
@@ -2789,7 +2756,7 @@
         <v>180</v>
       </c>
       <c r="B15" s="13">
-        <v>46175.36539417824</v>
+        <v>46180.050531064815</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>61</v>
@@ -2803,9 +2770,7 @@
       <c r="F15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
         <v>14</v>
       </c>
@@ -2824,7 +2789,7 @@
         <v>181</v>
       </c>
       <c r="B16" s="13">
-        <v>46176.81027090277</v>
+        <v>46180.050552326386</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>67</v>
@@ -2838,9 +2803,7 @@
       <c r="F16" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G16" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G16" s="10"/>
       <c r="H16" s="10" t="s">
         <v>34</v>
       </c>
@@ -2859,7 +2822,7 @@
         <v>182</v>
       </c>
       <c r="B17" s="13">
-        <v>46176.897516701385</v>
+        <v>46180.05057877315</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>73</v>
@@ -2873,9 +2836,7 @@
       <c r="F17" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G17" s="10"/>
       <c r="H17" s="10" t="s">
         <v>34</v>
       </c>
@@ -2894,7 +2855,7 @@
         <v>183</v>
       </c>
       <c r="B18" s="13">
-        <v>46176.89797092593</v>
+        <v>46180.050595821755</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>77</v>
@@ -2908,9 +2869,7 @@
       <c r="F18" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="G18" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G18" s="10"/>
       <c r="H18" s="10" t="s">
         <v>14</v>
       </c>
@@ -2926,7 +2885,7 @@
         <v>184</v>
       </c>
       <c r="B19" s="13">
-        <v>46176.9001487037</v>
+        <v>46180.05061259259</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>73</v>
@@ -2940,9 +2899,7 @@
       <c r="F19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G19" s="10"/>
       <c r="H19" s="10" t="s">
         <v>34</v>
       </c>
@@ -2961,7 +2918,7 @@
         <v>185</v>
       </c>
       <c r="B20" s="13">
-        <v>46176.98599523148</v>
+        <v>46180.050628576384</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>67</v>
@@ -2975,9 +2932,7 @@
       <c r="F20" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G20" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G20" s="10"/>
       <c r="H20" s="10" t="s">
         <v>34</v>
       </c>
@@ -2993,7 +2948,7 @@
         <v>186</v>
       </c>
       <c r="B21" s="13">
-        <v>46177.15724104167</v>
+        <v>46180.05064469908</v>
       </c>
       <c r="C21" s="10" t="s">
         <v>85</v>
@@ -3007,9 +2962,7 @@
       <c r="F21" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G21" s="10"/>
       <c r="H21" s="10" t="s">
         <v>14</v>
       </c>
@@ -3025,7 +2978,7 @@
         <v>187</v>
       </c>
       <c r="B22" s="13">
-        <v>46177.92069255787</v>
+        <v>46180.050660416666</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>46</v>
@@ -3039,9 +2992,7 @@
       <c r="F22" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G22" s="10"/>
       <c r="H22" s="10" t="s">
         <v>16</v>
       </c>
@@ -3057,7 +3008,7 @@
         <v>188</v>
       </c>
       <c r="B23" s="13">
-        <v>46177.94379626158</v>
+        <v>46180.050675833336</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>91</v>
@@ -3071,9 +3022,7 @@
       <c r="F23" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G23" s="10"/>
       <c r="H23" s="10" t="s">
         <v>14</v>
       </c>
@@ -3092,7 +3041,7 @@
         <v>189</v>
       </c>
       <c r="B24" s="13">
-        <v>46177.95516053241</v>
+        <v>46180.050692060184</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>95</v>
@@ -3106,9 +3055,7 @@
       <c r="F24" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G24" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G24" s="10"/>
       <c r="H24" s="10" t="s">
         <v>16</v>
       </c>
@@ -3127,7 +3074,7 @@
         <v>190</v>
       </c>
       <c r="B25" s="13">
-        <v>46178.09025260417</v>
+        <v>46180.05070755787</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>100</v>
@@ -3141,9 +3088,7 @@
       <c r="F25" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="G25" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G25" s="10"/>
       <c r="H25" s="10" t="s">
         <v>44</v>
       </c>
@@ -3159,7 +3104,7 @@
         <v>191</v>
       </c>
       <c r="B26" s="13">
-        <v>46179.0225042824</v>
+        <v>46180.05072400463</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>77</v>
@@ -3173,9 +3118,7 @@
       <c r="F26" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G26" s="10"/>
       <c r="H26" s="10" t="s">
         <v>14</v>
       </c>
@@ -3191,7 +3134,7 @@
         <v>192</v>
       </c>
       <c r="B27" s="13">
-        <v>46180.02262467593</v>
+        <v>46180.05074019676</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>105</v>
@@ -3202,9 +3145,7 @@
       <c r="F27" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="G27" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G27" s="10"/>
       <c r="H27" s="10" t="s">
         <v>16</v>
       </c>
@@ -3223,7 +3164,7 @@
         <v>193</v>
       </c>
       <c r="B28" s="13">
-        <v>46180.0250299537</v>
+        <v>46180.0507569676</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>105</v>
@@ -3234,9 +3175,7 @@
       <c r="F28" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="G28" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G28" s="10"/>
       <c r="H28" s="10" t="s">
         <v>14</v>
       </c>
@@ -3255,7 +3194,7 @@
         <v>194</v>
       </c>
       <c r="B29" s="13">
-        <v>46180.03628767361</v>
+        <v>46180.05077884259</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>105</v>
@@ -3266,9 +3205,7 @@
       <c r="F29" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="G29" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G29" s="10"/>
       <c r="H29" s="10" t="s">
         <v>14</v>
       </c>
@@ -3283,33 +3220,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="B30" s="13">
-        <v>46152.4115727662</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="H30" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q30" s="10" t="s">
-        <v>166</v>
-      </c>
+      <c r="A30" s="10"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="Q30" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3357,69 +3276,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>198</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>199</v>
       </c>
       <c r="E1" s="16" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G1" s="16" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="K1" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="L1" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="M1" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="N1" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="P1" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="Q1" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="R1" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="S1" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="T1" s="16" t="s">
         <v>211</v>
-      </c>
-      <c r="T1" s="16" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3448,7 +3367,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3458,7 +3377,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -11583,7 +11502,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C1" s="16" t="s">
         <v>5</v>
@@ -11592,7 +11511,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2">
@@ -11603,13 +11522,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D2" s="18" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -11626,7 +11545,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4">
@@ -11634,7 +11553,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>13</v>
@@ -11643,12 +11562,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>54</v>
@@ -11660,7 +11579,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6">
@@ -11692,25 +11611,25 @@
         <v>16</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>223</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13">
@@ -11720,17 +11639,17 @@
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17">
@@ -11740,12 +11659,12 @@
     </row>
     <row r="18">
       <c r="B18" s="18" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20">
@@ -11760,7 +11679,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -11770,7 +11689,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v11 2026-06-07 15:29 IST
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="252">
   <si>
     <t>Timestamp</t>
   </si>
@@ -398,6 +398,27 @@
     <t>https://drive.google.com/open?id=1YFsB7fzGaMal0KqGORwHUyyKLc2jw8-f</t>
   </si>
   <si>
+    <t>Waterproofing</t>
+  </si>
+  <si>
+    <t>Re-do waterproofing on façade areas — leakage observed during rain; not properly done. The black glue (bituminous sealant) must be applied properly.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1abBMZP2_wqw7qLHKRxil35mxwkiajgYP, https://drive.google.com/open?id=18yaRZJQROfD4wr2iNTGM6xmbzSnuP9Fv</t>
+  </si>
+  <si>
+    <t>Apply anti-rust primer / paint on all metal surfaces (railings, grills, STP area grills) before final painting. Applicable across the society.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1RCvFn355x9hgINOxX6WAP4DpibN_Oczb, https://drive.google.com/open?id=1FEeNUIMdHn1cq_WYDxVFhvpDXFgsVVld</t>
+  </si>
+  <si>
+    <t>Provide proper frame casing / conduits for all exposed wiring. Electrical – Wire casing / conduits. Applicable for Pump Area, Electrical Meter area all three towers, Parking Roofs</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1IR0u7kWCk_6yiKLyksszpHj28VsPgudk</t>
+  </si>
+  <si>
     <t>Key</t>
   </si>
   <si>
@@ -635,6 +656,18 @@
     <t>TKT-00029</t>
   </si>
   <si>
+    <t>TKT-00030</t>
+  </si>
+  <si>
+    <t>TKT-00031</t>
+  </si>
+  <si>
+    <t>TKT-00032</t>
+  </si>
+  <si>
+    <t>TKT-00033</t>
+  </si>
+  <si>
     <t>TA-0001</t>
   </si>
   <si>
@@ -702,9 +735,6 @@
   </si>
   <si>
     <t>VERIFIED</t>
-  </si>
-  <si>
-    <t>Waterproofing</t>
   </si>
   <si>
     <t>Fire Safety</t>
@@ -970,7 +1000,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I34" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I37" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="9">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Resident Name" id="2"/>
@@ -2015,6 +2045,75 @@
         <v>124</v>
       </c>
     </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="6">
+        <v>46180.110090902774</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="6">
+        <v>46180.11527789352</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="6">
+        <v>46180.12016730324</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="I37" s="8" t="s">
+        <v>131</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I15"/>
@@ -2027,10 +2126,11 @@
     <hyperlink r:id="rId8" ref="I31"/>
     <hyperlink r:id="rId9" ref="I32"/>
     <hyperlink r:id="rId10" ref="I34"/>
+    <hyperlink r:id="rId11" ref="I37"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId12"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2049,369 +2149,369 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B6" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B7" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B8" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B9" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B10" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B11" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B12" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B13" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B14" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="B15" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B16" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B17" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B18" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="B19" s="10">
         <v>20.0</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B20" s="10">
         <v>20.0</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B21" s="10">
         <v>5.0</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B22" s="10">
         <v>5.0</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B23" s="10">
         <v>1600.0</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B24" s="10">
         <v>0.85</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B25" s="10">
         <v>5.0</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B26" s="10">
         <v>1000.0</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B27" s="10">
         <v>300.0</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B32" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="10" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2436,7 +2536,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B1" s="13">
         <v>46151.165393194446</v>
@@ -2463,18 +2563,18 @@
         <v>15</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B2" s="13">
-        <v>46180.05029387731</v>
+        <v>46180.10313505787</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>9</v>
@@ -2501,15 +2601,15 @@
       <c r="L2" s="14"/>
       <c r="M2" s="10"/>
       <c r="Q2" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B3" s="13">
-        <v>46180.05031049768</v>
+        <v>46180.10315137732</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>9</v>
@@ -2531,15 +2631,15 @@
       </c>
       <c r="K3" s="10"/>
       <c r="Q3" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B4" s="13">
-        <v>46180.050328125</v>
+        <v>46180.103169236114</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>9</v>
@@ -2564,15 +2664,15 @@
       </c>
       <c r="K4" s="10"/>
       <c r="Q4" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B5" s="13">
-        <v>46180.05034636574</v>
+        <v>46180.10318601852</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>9</v>
@@ -2597,15 +2697,15 @@
       </c>
       <c r="K5" s="10"/>
       <c r="Q5" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B6" s="13">
-        <v>46180.0503632176</v>
+        <v>46180.103206631946</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>30</v>
@@ -2630,15 +2730,15 @@
       </c>
       <c r="K6" s="10"/>
       <c r="Q6" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B7" s="13">
-        <v>46180.05037993056</v>
+        <v>46180.10322395833</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>9</v>
@@ -2660,15 +2760,15 @@
       </c>
       <c r="K7" s="10"/>
       <c r="Q7" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B8" s="13">
-        <v>46180.050404814814</v>
+        <v>46180.103242303245</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>9</v>
@@ -2688,15 +2788,15 @@
       </c>
       <c r="K8" s="10"/>
       <c r="Q8" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B9" s="13">
-        <v>46180.05042226852</v>
+        <v>46180.103259386575</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>41</v>
@@ -2718,15 +2818,15 @@
         <v>45</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B10" s="13">
-        <v>46180.05044378473</v>
+        <v>46180.103281620366</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>46</v>
@@ -2748,15 +2848,15 @@
         <v>49</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B11" s="13">
-        <v>46180.05046524305</v>
+        <v>46180.10330618055</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>50</v>
@@ -2778,15 +2878,15 @@
         <v>53</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B12" s="13">
-        <v>46180.050481909726</v>
+        <v>46180.10332761574</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>30</v>
@@ -2808,15 +2908,15 @@
         <v>55</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B13" s="13">
-        <v>46180.05049804398</v>
+        <v>46180.10334641204</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>56</v>
@@ -2841,15 +2941,15 @@
         <v>59</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B14" s="13">
-        <v>46180.05051513889</v>
+        <v>46180.103362615744</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>61</v>
@@ -2874,15 +2974,15 @@
         <v>63</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B15" s="13">
-        <v>46180.050531064815</v>
+        <v>46180.10338010416</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>61</v>
@@ -2907,15 +3007,15 @@
         <v>65</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B16" s="13">
-        <v>46180.050552326386</v>
+        <v>46180.10339710648</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>67</v>
@@ -2940,15 +3040,15 @@
         <v>71</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B17" s="13">
-        <v>46180.05057877315</v>
+        <v>46180.10341520833</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>73</v>
@@ -2973,15 +3073,15 @@
         <v>75</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B18" s="13">
-        <v>46180.050595821755</v>
+        <v>46180.10343418982</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>77</v>
@@ -3003,15 +3103,15 @@
         <v>80</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B19" s="13">
-        <v>46180.05061259259</v>
+        <v>46180.10344982639</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>73</v>
@@ -3036,15 +3136,15 @@
         <v>82</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B20" s="13">
-        <v>46180.050628576384</v>
+        <v>46180.103465231485</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>67</v>
@@ -3066,15 +3166,15 @@
         <v>84</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B21" s="13">
-        <v>46180.05064469908</v>
+        <v>46180.103480879625</v>
       </c>
       <c r="C21" s="10" t="s">
         <v>85</v>
@@ -3096,15 +3196,15 @@
         <v>87</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="B22" s="13">
-        <v>46180.050660416666</v>
+        <v>46180.103501053236</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>46</v>
@@ -3126,15 +3226,15 @@
         <v>90</v>
       </c>
       <c r="Q22" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B23" s="13">
-        <v>46180.050675833336</v>
+        <v>46180.10351888889</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>91</v>
@@ -3159,15 +3259,15 @@
         <v>93</v>
       </c>
       <c r="Q23" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="B24" s="13">
-        <v>46180.050692060184</v>
+        <v>46180.103536608796</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>95</v>
@@ -3192,15 +3292,15 @@
         <v>98</v>
       </c>
       <c r="Q24" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B25" s="13">
-        <v>46180.05070755787</v>
+        <v>46180.103555381946</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>100</v>
@@ -3222,15 +3322,15 @@
         <v>102</v>
       </c>
       <c r="Q25" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B26" s="13">
-        <v>46180.05072400463</v>
+        <v>46180.10357407408</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>77</v>
@@ -3252,15 +3352,15 @@
         <v>104</v>
       </c>
       <c r="Q26" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B27" s="13">
-        <v>46180.05074019676</v>
+        <v>46180.103594050925</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>105</v>
@@ -3282,15 +3382,15 @@
         <v>107</v>
       </c>
       <c r="Q27" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B28" s="13">
-        <v>46180.0507569676</v>
+        <v>46180.10361086806</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>105</v>
@@ -3312,15 +3412,15 @@
         <v>110</v>
       </c>
       <c r="Q28" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B29" s="13">
-        <v>46180.05077884259</v>
+        <v>46180.10362674769</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>105</v>
@@ -3342,15 +3442,15 @@
         <v>113</v>
       </c>
       <c r="Q29" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B30" s="13">
-        <v>46180.065786956024</v>
+        <v>46180.10364325231</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>105</v>
@@ -3362,9 +3462,7 @@
       <c r="F30" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G30" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G30" s="10"/>
       <c r="H30" s="10" t="s">
         <v>16</v>
       </c>
@@ -3375,15 +3473,15 @@
         <v>115</v>
       </c>
       <c r="Q30" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B31" s="13">
-        <v>46180.09252373842</v>
+        <v>46180.10365928241</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>105</v>
@@ -3394,9 +3492,7 @@
       <c r="F31" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G31" s="10"/>
       <c r="H31" s="10" t="s">
         <v>16</v>
       </c>
@@ -3407,15 +3503,15 @@
         <v>118</v>
       </c>
       <c r="Q31" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="B32" s="13">
-        <v>46180.09559391203</v>
+        <v>46180.10367861111</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>105</v>
@@ -3426,9 +3522,7 @@
       <c r="F32" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="G32" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G32" s="10"/>
       <c r="H32" s="10" t="s">
         <v>16</v>
       </c>
@@ -3436,15 +3530,15 @@
         <v>121</v>
       </c>
       <c r="Q32" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="B33" s="13">
-        <v>46180.09867041667</v>
+        <v>46180.103699074076</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>105</v>
@@ -3455,9 +3549,7 @@
       <c r="F33" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="G33" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="G33" s="10"/>
       <c r="H33" s="10" t="s">
         <v>16</v>
       </c>
@@ -3468,7 +3560,103 @@
         <v>123</v>
       </c>
       <c r="Q33" s="10" t="s">
-        <v>175</v>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B34" s="13">
+        <v>46180.11010986111</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="J34" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q34" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B35" s="13">
+        <v>46180.11529725694</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="J35" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q35" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="B36" s="13">
+        <v>46180.1201821412</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I36" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="J36" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q36" s="10" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -3483,8 +3671,9 @@
     <hyperlink r:id="rId8" ref="I30"/>
     <hyperlink r:id="rId9" ref="I31"/>
     <hyperlink r:id="rId10" ref="I33"/>
+    <hyperlink r:id="rId11" ref="I36"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
 
@@ -3520,69 +3709,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="G1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="I1" s="15" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="Q1" s="15" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3611,7 +3800,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3621,7 +3810,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -11746,7 +11935,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>5</v>
@@ -11755,7 +11944,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2">
@@ -11766,13 +11955,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3">
@@ -11789,7 +11978,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4">
@@ -11797,7 +11986,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>227</v>
+        <v>125</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>13</v>
@@ -11806,12 +11995,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>54</v>
@@ -11823,7 +12012,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6">
@@ -11855,25 +12044,25 @@
         <v>16</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
@@ -11883,17 +12072,17 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17">
@@ -11903,12 +12092,12 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20">
@@ -11923,7 +12112,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="17" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -11933,7 +12122,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="17" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v12 2026-06-07 15:32 IST
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="257">
   <si>
     <t>Timestamp</t>
   </si>
@@ -419,6 +419,15 @@
     <t>https://drive.google.com/open?id=1IR0u7kWCk_6yiKLyksszpHj28VsPgudk</t>
   </si>
   <si>
+    <t>Earthing</t>
+  </si>
+  <si>
+    <t>Provide casing for open earthing wires. Observed at the new C-Wing stack parking adjacent to the C-Wing interior entrance.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1sOoR2P0OSlyM1Hv81a5NY7q9N9Kk48SG</t>
+  </si>
+  <si>
     <t>Key</t>
   </si>
   <si>
@@ -668,6 +677,15 @@
     <t>TKT-00033</t>
   </si>
   <si>
+    <t>TKT-00034</t>
+  </si>
+  <si>
+    <t>TKT-00035</t>
+  </si>
+  <si>
+    <t>TKT-00036</t>
+  </si>
+  <si>
     <t>TA-0001</t>
   </si>
   <si>
@@ -747,9 +765,6 @@
   </si>
   <si>
     <t>Documentation</t>
-  </si>
-  <si>
-    <t>Earthing</t>
   </si>
   <si>
     <t>Switch Issue</t>
@@ -1000,7 +1015,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I37" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I38" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="9">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Resident Name" id="2"/>
@@ -2114,6 +2129,29 @@
         <v>131</v>
       </c>
     </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="6">
+        <v>46180.12603246528</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>134</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I15"/>
@@ -2127,10 +2165,11 @@
     <hyperlink r:id="rId9" ref="I32"/>
     <hyperlink r:id="rId10" ref="I34"/>
     <hyperlink r:id="rId11" ref="I37"/>
+    <hyperlink r:id="rId12" ref="I38"/>
   </hyperlinks>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId13"/>
   <tableParts count="1">
-    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2149,369 +2188,369 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B6" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B7" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B8" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B9" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B10" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B11" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B12" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B13" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B14" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B15" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B16" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B17" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B18" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B19" s="10">
         <v>20.0</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B20" s="10">
         <v>20.0</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B21" s="10">
         <v>5.0</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B22" s="10">
         <v>5.0</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B23" s="10">
         <v>1600.0</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B24" s="10">
         <v>0.85</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B25" s="10">
         <v>5.0</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B26" s="10">
         <v>1000.0</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B27" s="10">
         <v>300.0</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B32" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2536,7 +2575,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B1" s="13">
         <v>46151.165393194446</v>
@@ -2563,15 +2602,15 @@
         <v>15</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B2" s="13">
         <v>46180.10313505787</v>
@@ -2601,12 +2640,12 @@
       <c r="L2" s="14"/>
       <c r="M2" s="10"/>
       <c r="Q2" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B3" s="13">
         <v>46180.10315137732</v>
@@ -2631,12 +2670,12 @@
       </c>
       <c r="K3" s="10"/>
       <c r="Q3" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B4" s="13">
         <v>46180.103169236114</v>
@@ -2664,12 +2703,12 @@
       </c>
       <c r="K4" s="10"/>
       <c r="Q4" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B5" s="13">
         <v>46180.10318601852</v>
@@ -2697,12 +2736,12 @@
       </c>
       <c r="K5" s="10"/>
       <c r="Q5" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B6" s="13">
         <v>46180.103206631946</v>
@@ -2730,12 +2769,12 @@
       </c>
       <c r="K6" s="10"/>
       <c r="Q6" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B7" s="13">
         <v>46180.10322395833</v>
@@ -2760,12 +2799,12 @@
       </c>
       <c r="K7" s="10"/>
       <c r="Q7" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B8" s="13">
         <v>46180.103242303245</v>
@@ -2788,12 +2827,12 @@
       </c>
       <c r="K8" s="10"/>
       <c r="Q8" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B9" s="13">
         <v>46180.103259386575</v>
@@ -2818,12 +2857,12 @@
         <v>45</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B10" s="13">
         <v>46180.103281620366</v>
@@ -2848,12 +2887,12 @@
         <v>49</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B11" s="13">
         <v>46180.10330618055</v>
@@ -2878,12 +2917,12 @@
         <v>53</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B12" s="13">
         <v>46180.10332761574</v>
@@ -2908,12 +2947,12 @@
         <v>55</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B13" s="13">
         <v>46180.10334641204</v>
@@ -2941,12 +2980,12 @@
         <v>59</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B14" s="13">
         <v>46180.103362615744</v>
@@ -2974,12 +3013,12 @@
         <v>63</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B15" s="13">
         <v>46180.10338010416</v>
@@ -3007,12 +3046,12 @@
         <v>65</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B16" s="13">
         <v>46180.10339710648</v>
@@ -3040,12 +3079,12 @@
         <v>71</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B17" s="13">
         <v>46180.10341520833</v>
@@ -3073,12 +3112,12 @@
         <v>75</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B18" s="13">
         <v>46180.10343418982</v>
@@ -3103,12 +3142,12 @@
         <v>80</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B19" s="13">
         <v>46180.10344982639</v>
@@ -3136,12 +3175,12 @@
         <v>82</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B20" s="13">
         <v>46180.103465231485</v>
@@ -3166,12 +3205,12 @@
         <v>84</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B21" s="13">
         <v>46180.103480879625</v>
@@ -3196,12 +3235,12 @@
         <v>87</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B22" s="13">
         <v>46180.103501053236</v>
@@ -3226,12 +3265,12 @@
         <v>90</v>
       </c>
       <c r="Q22" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B23" s="13">
         <v>46180.10351888889</v>
@@ -3259,12 +3298,12 @@
         <v>93</v>
       </c>
       <c r="Q23" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B24" s="13">
         <v>46180.103536608796</v>
@@ -3292,12 +3331,12 @@
         <v>98</v>
       </c>
       <c r="Q24" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B25" s="13">
         <v>46180.103555381946</v>
@@ -3322,12 +3361,12 @@
         <v>102</v>
       </c>
       <c r="Q25" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B26" s="13">
         <v>46180.10357407408</v>
@@ -3352,12 +3391,12 @@
         <v>104</v>
       </c>
       <c r="Q26" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B27" s="13">
         <v>46180.103594050925</v>
@@ -3382,12 +3421,12 @@
         <v>107</v>
       </c>
       <c r="Q27" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B28" s="13">
         <v>46180.10361086806</v>
@@ -3412,12 +3451,12 @@
         <v>110</v>
       </c>
       <c r="Q28" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B29" s="13">
         <v>46180.10362674769</v>
@@ -3442,12 +3481,12 @@
         <v>113</v>
       </c>
       <c r="Q29" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B30" s="13">
         <v>46180.10364325231</v>
@@ -3473,12 +3512,12 @@
         <v>115</v>
       </c>
       <c r="Q30" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B31" s="13">
         <v>46180.10365928241</v>
@@ -3503,12 +3542,12 @@
         <v>118</v>
       </c>
       <c r="Q31" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B32" s="13">
         <v>46180.10367861111</v>
@@ -3530,12 +3569,12 @@
         <v>121</v>
       </c>
       <c r="Q32" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B33" s="13">
         <v>46180.103699074076</v>
@@ -3560,12 +3599,12 @@
         <v>123</v>
       </c>
       <c r="Q33" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B34" s="13">
         <v>46180.11010986111</v>
@@ -3592,12 +3631,12 @@
         <v>126</v>
       </c>
       <c r="Q34" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B35" s="13">
         <v>46180.11529725694</v>
@@ -3624,12 +3663,12 @@
         <v>128</v>
       </c>
       <c r="Q35" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B36" s="13">
         <v>46180.1201821412</v>
@@ -3656,7 +3695,39 @@
         <v>130</v>
       </c>
       <c r="Q36" s="10" t="s">
-        <v>182</v>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B37" s="13">
+        <v>46180.12604854167</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I37" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="J37" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q37" s="10" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -3672,8 +3743,9 @@
     <hyperlink r:id="rId9" ref="I31"/>
     <hyperlink r:id="rId10" ref="I33"/>
     <hyperlink r:id="rId11" ref="I36"/>
+    <hyperlink r:id="rId12" ref="I37"/>
   </hyperlinks>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
 
@@ -3709,69 +3781,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="G1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="I1" s="15" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="Q1" s="15" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3800,7 +3872,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3810,7 +3882,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -11935,7 +12007,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>5</v>
@@ -11944,7 +12016,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2">
@@ -11955,13 +12027,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3">
@@ -11978,7 +12050,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4">
@@ -11995,12 +12067,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>54</v>
@@ -12012,7 +12084,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6">
@@ -12044,25 +12116,25 @@
         <v>16</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>242</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13">
@@ -12072,17 +12144,17 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="17">
@@ -12092,12 +12164,12 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20">
@@ -12112,7 +12184,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="17" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -12122,7 +12194,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="17" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v13 2026-06-07 15:56 IST
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="260">
   <si>
     <t>Timestamp</t>
   </si>
@@ -428,6 +428,12 @@
     <t>https://drive.google.com/open?id=1sOoR2P0OSlyM1Hv81a5NY7q9N9Kk48SG</t>
   </si>
   <si>
+    <t>Seal and finish all electrical cable entry points into the building.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1IiGMXrLYuGTzW8OPFrgr-2scpv8jbdZX, https://drive.google.com/open?id=1NkjmfuzIIF99lpJMT_mwgeuz52jlDhvi, https://drive.google.com/open?id=10IPjCesav19m7N0xVkGDpJkShavsqMgT, https://drive.google.com/open?id=1G0GGnId09yBbwqJ5yD7_PDzUbiWFkFfo</t>
+  </si>
+  <si>
     <t>Key</t>
   </si>
   <si>
@@ -684,6 +690,9 @@
   </si>
   <si>
     <t>TKT-00036</t>
+  </si>
+  <si>
+    <t>TKT-00037</t>
   </si>
   <si>
     <t>TA-0001</t>
@@ -1015,7 +1024,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I38" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I39" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="9">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Resident Name" id="2"/>
@@ -2152,6 +2161,29 @@
         <v>134</v>
       </c>
     </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="6">
+        <v>46180.1336691551</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I15"/>
@@ -2188,369 +2220,369 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>139</v>
-      </c>
       <c r="C3" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B6" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B8" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B9" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B10" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B11" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B12" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B13" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B14" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B15" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B16" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B17" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B18" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B19" s="10">
         <v>20.0</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B20" s="10">
         <v>20.0</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B21" s="10">
         <v>5.0</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B22" s="10">
         <v>5.0</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B23" s="10">
         <v>1600.0</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B24" s="10">
         <v>0.85</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B25" s="10">
         <v>5.0</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B26" s="10">
         <v>1000.0</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B27" s="10">
         <v>300.0</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B32" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2575,7 +2607,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B1" s="13">
         <v>46151.165393194446</v>
@@ -2602,15 +2634,15 @@
         <v>15</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B2" s="13">
         <v>46180.10313505787</v>
@@ -2640,12 +2672,12 @@
       <c r="L2" s="14"/>
       <c r="M2" s="10"/>
       <c r="Q2" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B3" s="13">
         <v>46180.10315137732</v>
@@ -2670,12 +2702,12 @@
       </c>
       <c r="K3" s="10"/>
       <c r="Q3" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B4" s="13">
         <v>46180.103169236114</v>
@@ -2703,12 +2735,12 @@
       </c>
       <c r="K4" s="10"/>
       <c r="Q4" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B5" s="13">
         <v>46180.10318601852</v>
@@ -2736,12 +2768,12 @@
       </c>
       <c r="K5" s="10"/>
       <c r="Q5" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B6" s="13">
         <v>46180.103206631946</v>
@@ -2769,12 +2801,12 @@
       </c>
       <c r="K6" s="10"/>
       <c r="Q6" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B7" s="13">
         <v>46180.10322395833</v>
@@ -2799,12 +2831,12 @@
       </c>
       <c r="K7" s="10"/>
       <c r="Q7" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B8" s="13">
         <v>46180.103242303245</v>
@@ -2827,12 +2859,12 @@
       </c>
       <c r="K8" s="10"/>
       <c r="Q8" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B9" s="13">
         <v>46180.103259386575</v>
@@ -2857,12 +2889,12 @@
         <v>45</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B10" s="13">
         <v>46180.103281620366</v>
@@ -2887,12 +2919,12 @@
         <v>49</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B11" s="13">
         <v>46180.10330618055</v>
@@ -2917,12 +2949,12 @@
         <v>53</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B12" s="13">
         <v>46180.10332761574</v>
@@ -2947,12 +2979,12 @@
         <v>55</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B13" s="13">
         <v>46180.10334641204</v>
@@ -2980,12 +3012,12 @@
         <v>59</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B14" s="13">
         <v>46180.103362615744</v>
@@ -3013,12 +3045,12 @@
         <v>63</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B15" s="13">
         <v>46180.10338010416</v>
@@ -3046,12 +3078,12 @@
         <v>65</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B16" s="13">
         <v>46180.10339710648</v>
@@ -3079,12 +3111,12 @@
         <v>71</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B17" s="13">
         <v>46180.10341520833</v>
@@ -3112,12 +3144,12 @@
         <v>75</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B18" s="13">
         <v>46180.10343418982</v>
@@ -3142,12 +3174,12 @@
         <v>80</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B19" s="13">
         <v>46180.10344982639</v>
@@ -3175,12 +3207,12 @@
         <v>82</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B20" s="13">
         <v>46180.103465231485</v>
@@ -3205,12 +3237,12 @@
         <v>84</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B21" s="13">
         <v>46180.103480879625</v>
@@ -3235,12 +3267,12 @@
         <v>87</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B22" s="13">
         <v>46180.103501053236</v>
@@ -3265,12 +3297,12 @@
         <v>90</v>
       </c>
       <c r="Q22" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B23" s="13">
         <v>46180.10351888889</v>
@@ -3298,12 +3330,12 @@
         <v>93</v>
       </c>
       <c r="Q23" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B24" s="13">
         <v>46180.103536608796</v>
@@ -3331,12 +3363,12 @@
         <v>98</v>
       </c>
       <c r="Q24" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B25" s="13">
         <v>46180.103555381946</v>
@@ -3361,12 +3393,12 @@
         <v>102</v>
       </c>
       <c r="Q25" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B26" s="13">
         <v>46180.10357407408</v>
@@ -3391,12 +3423,12 @@
         <v>104</v>
       </c>
       <c r="Q26" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B27" s="13">
         <v>46180.103594050925</v>
@@ -3421,12 +3453,12 @@
         <v>107</v>
       </c>
       <c r="Q27" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B28" s="13">
         <v>46180.10361086806</v>
@@ -3451,12 +3483,12 @@
         <v>110</v>
       </c>
       <c r="Q28" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B29" s="13">
         <v>46180.10362674769</v>
@@ -3481,12 +3513,12 @@
         <v>113</v>
       </c>
       <c r="Q29" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B30" s="13">
         <v>46180.10364325231</v>
@@ -3512,12 +3544,12 @@
         <v>115</v>
       </c>
       <c r="Q30" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B31" s="13">
         <v>46180.10365928241</v>
@@ -3542,12 +3574,12 @@
         <v>118</v>
       </c>
       <c r="Q31" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B32" s="13">
         <v>46180.10367861111</v>
@@ -3569,12 +3601,12 @@
         <v>121</v>
       </c>
       <c r="Q32" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B33" s="13">
         <v>46180.103699074076</v>
@@ -3599,12 +3631,12 @@
         <v>123</v>
       </c>
       <c r="Q33" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B34" s="13">
         <v>46180.11010986111</v>
@@ -3631,12 +3663,12 @@
         <v>126</v>
       </c>
       <c r="Q34" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B35" s="13">
         <v>46180.11529725694</v>
@@ -3663,12 +3695,12 @@
         <v>128</v>
       </c>
       <c r="Q35" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B36" s="13">
         <v>46180.1201821412</v>
@@ -3695,12 +3727,12 @@
         <v>130</v>
       </c>
       <c r="Q36" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B37" s="13">
         <v>46180.12604854167</v>
@@ -3727,7 +3759,39 @@
         <v>133</v>
       </c>
       <c r="Q37" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="B38" s="13">
+        <v>46180.133690347226</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="J38" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q38" s="10" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -3781,69 +3845,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I1" s="15" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="Q1" s="15" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3872,7 +3936,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3882,7 +3946,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -12007,7 +12071,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>5</v>
@@ -12016,7 +12080,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2">
@@ -12027,13 +12091,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
@@ -12050,7 +12114,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4">
@@ -12067,12 +12131,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>54</v>
@@ -12084,7 +12148,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6">
@@ -12116,12 +12180,12 @@
         <v>16</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>132</v>
@@ -12129,12 +12193,12 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="13">
@@ -12144,17 +12208,17 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17">
@@ -12164,12 +12228,12 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="20">
@@ -12184,7 +12248,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="17" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -12194,7 +12258,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="17" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v14 2026-06-08 02:29 IST [weekly]
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="311">
   <si>
     <t>Timestamp</t>
   </si>
@@ -434,6 +434,111 @@
     <t>https://drive.google.com/open?id=1IiGMXrLYuGTzW8OPFrgr-2scpv8jbdZX, https://drive.google.com/open?id=1NkjmfuzIIF99lpJMT_mwgeuz52jlDhvi, https://drive.google.com/open?id=10IPjCesav19m7N0xVkGDpJkShavsqMgT, https://drive.google.com/open?id=1G0GGnId09yBbwqJ5yD7_PDzUbiWFkFfo</t>
   </si>
   <si>
+    <t>Complete painting of the C-Wing and Main Entrance storage rooms. Storage room painting. At C wing and Main Enterance</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Fbucuw-dd_GGnbe2xvOO49LWOElNl3Jd, https://drive.google.com/open?id=1ywbs655JHfoTTRn8R2A7UMcnDznKucRr</t>
+  </si>
+  <si>
+    <t>Assessment 6th June</t>
+  </si>
+  <si>
+    <t>Pool toilet – Wall holes / paint - Two holes at the pool toilet to be filled &amp; painted.</t>
+  </si>
+  <si>
+    <t>Civil – Broken ceiling support - Broken ceiling support to be repaired.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Voq6jwE626Z12uMVNPiDWNo7G8AsEk9Q</t>
+  </si>
+  <si>
+    <t>Broken tiles and unfinished civil work in the space — fix.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1NoaIg2OGMY0_VrLryiSi3XWPJu_4yldM</t>
+  </si>
+  <si>
+    <t>Electric light hanging on one side, broken — lower basement below B-Wing. Re-fix.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Ba5nXQXIZQF1WzPwRb4J_gRoFfZWKXn7</t>
+  </si>
+  <si>
+    <t>Open grills at the pillar in the lower basement — risky; close them.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1SCtj3xVhgvIAXpt8JNUQ3SRHfKyL_UC5</t>
+  </si>
+  <si>
+    <t>Staircase to the garden area from A-Building has been removed; people may attempt to jump — install a barrier / restore the staircase.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Kxg3p7ymQlKlBrzMRLsIgL-4_y13-dMv</t>
+  </si>
+  <si>
+    <t>Switch Issue</t>
+  </si>
+  <si>
+    <t>Sockets are of poor quality and at a height accessible to children — relocate / upgrade them, or provide a protective cover / guard.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=12BhqPkmBHBBMOMbSKR8lt4F8LdiNSGBg</t>
+  </si>
+  <si>
+    <t>Grouting must be fixed at all locations before painting is done.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1l_cc95APL57piXSumyn7aTDE1VCY3je5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assessment 6th June </t>
+  </si>
+  <si>
+    <t>Apply rubber paint / anti-skid coating on all driveways — ground floor and lower basement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passage access and cleanliness </t>
+  </si>
+  <si>
+    <t>"Strengthen the access / passage between the (A ↔ B ↔ C) wing ducts. A sturdy 20 ft ladder is required in order to establish a fortnightly cleaning schedule for the first-floor ducts between A–B, B–B and B–C, to maintain hygiene and health. • Cleaning to be carried out under supervision only. • Builder must get this cleaned before hand-over."</t>
+  </si>
+  <si>
+    <t>"External-wall painting to be done last, after all civil works are complete. • Covers all floor walls, refuge areas, and any patch-work. • All ducts must be left paan / stain-free."</t>
+  </si>
+  <si>
+    <t>Cleaning</t>
+  </si>
+  <si>
+    <t>"Carry out cleaning of the following before handover (mandatory): • Society water tank • Balancing tank • Swimming-pool tank"</t>
+  </si>
+  <si>
+    <t>Equipments</t>
+  </si>
+  <si>
+    <t>Hand over M2M (machine-to-machine / monitoring) system details for the Diesel Generator.</t>
+  </si>
+  <si>
+    <t>Provide warranty and guarantee certificates for the Diesel Generator.</t>
+  </si>
+  <si>
+    <t>Sync between Lift 1 &amp; 2</t>
+  </si>
+  <si>
+    <t>Lifts in A-Wing and C-Wing are not operating in sync. Configure synchronisation logic so that idle lifts are not called unnecessarily, thereby reducing energy consumption.</t>
+  </si>
+  <si>
+    <t>Door</t>
+  </si>
+  <si>
+    <t>Door of the STP should be locked, since it has open drains and is risky.</t>
+  </si>
+  <si>
+    <t>Cleaning of all the ducts and common areas</t>
+  </si>
+  <si>
+    <t>Proper cleaning is required since moslty its because of construction remains on.</t>
+  </si>
+  <si>
     <t>Key</t>
   </si>
   <si>
@@ -695,7 +800,61 @@
     <t>TKT-00037</t>
   </si>
   <si>
-    <t>TA-0001</t>
+    <t>TKT-00038</t>
+  </si>
+  <si>
+    <t>TKT-00039</t>
+  </si>
+  <si>
+    <t>TKT-00040</t>
+  </si>
+  <si>
+    <t>TKT-00041</t>
+  </si>
+  <si>
+    <t>TKT-00042</t>
+  </si>
+  <si>
+    <t>TKT-00043</t>
+  </si>
+  <si>
+    <t>TKT-00044</t>
+  </si>
+  <si>
+    <t>TKT-00045</t>
+  </si>
+  <si>
+    <t>TKT-00046</t>
+  </si>
+  <si>
+    <t>TKT-00047</t>
+  </si>
+  <si>
+    <t>TKT-00048</t>
+  </si>
+  <si>
+    <t>TKT-00049</t>
+  </si>
+  <si>
+    <t>TKT-00050</t>
+  </si>
+  <si>
+    <t>TKT-00051</t>
+  </si>
+  <si>
+    <t>TKT-00052</t>
+  </si>
+  <si>
+    <t>TKT-00053</t>
+  </si>
+  <si>
+    <t>TKT-00054</t>
+  </si>
+  <si>
+    <t>TKT-00055</t>
+  </si>
+  <si>
+    <t>TKT-00056</t>
   </si>
   <si>
     <t>Ticket ID</t>
@@ -776,16 +935,10 @@
     <t>Documentation</t>
   </si>
   <si>
-    <t>Switch Issue</t>
-  </si>
-  <si>
     <t>Alarm</t>
   </si>
   <si>
     <t>Sprinkler</t>
-  </si>
-  <si>
-    <t>Door</t>
   </si>
   <si>
     <t>Intercom</t>
@@ -1024,7 +1177,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I39" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I57" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="9">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Resident Name" id="2"/>
@@ -2184,6 +2337,441 @@
         <v>136</v>
       </c>
     </row>
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="6">
+        <v>46180.144973877315</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="41" ht="22.5" customHeight="1">
+      <c r="A41" s="6">
+        <v>46180.42401563657</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="42" ht="22.5" customHeight="1">
+      <c r="A42" s="6">
+        <v>46180.425612129635</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" ht="22.5" customHeight="1">
+      <c r="A43" s="6">
+        <v>46180.42675886574</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I43" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="44" ht="22.5" customHeight="1">
+      <c r="A44" s="6">
+        <v>46180.428417476855</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I44" s="8" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" ht="22.5" customHeight="1">
+      <c r="A45" s="6">
+        <v>46180.43109547454</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="I45" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="6">
+        <v>46180.48139981482</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I46" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="A47" s="6">
+        <v>46180.49303815972</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="A48" s="6">
+        <v>46180.49662355324</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I48" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="A49" s="6">
+        <v>46180.49831425926</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="50" ht="22.5" customHeight="1">
+      <c r="A50" s="6">
+        <v>46180.556043055556</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="51" ht="22.5" customHeight="1">
+      <c r="A51" s="6">
+        <v>46180.556593877314</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" ht="22.5" customHeight="1">
+      <c r="A52" s="6">
+        <v>46180.55721949074</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="53" ht="22.5" customHeight="1">
+      <c r="A53" s="6">
+        <v>46180.557835879634</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="54" ht="22.5" customHeight="1">
+      <c r="A54" s="6">
+        <v>46180.558336331014</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H54" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="55" ht="22.5" customHeight="1">
+      <c r="A55" s="6">
+        <v>46180.55919884259</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="56" ht="22.5" customHeight="1">
+      <c r="A56" s="6">
+        <v>46180.55975138889</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="57" ht="22.5" customHeight="1">
+      <c r="A57" s="6">
+        <v>46180.56035644676</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I15"/>
@@ -2198,10 +2786,17 @@
     <hyperlink r:id="rId10" ref="I34"/>
     <hyperlink r:id="rId11" ref="I37"/>
     <hyperlink r:id="rId12" ref="I38"/>
+    <hyperlink r:id="rId13" ref="I42"/>
+    <hyperlink r:id="rId14" ref="I43"/>
+    <hyperlink r:id="rId15" ref="I44"/>
+    <hyperlink r:id="rId16" ref="I45"/>
+    <hyperlink r:id="rId17" ref="I46"/>
+    <hyperlink r:id="rId18" ref="I47"/>
+    <hyperlink r:id="rId19" ref="I48"/>
   </hyperlinks>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId20"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId22"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2220,369 +2815,369 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>137</v>
+        <v>172</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>138</v>
+        <v>173</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>139</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>141</v>
+        <v>176</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>142</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>143</v>
+        <v>178</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>141</v>
+        <v>176</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>145</v>
+        <v>180</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>146</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>147</v>
+        <v>182</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>148</v>
+        <v>183</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="B6" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>152</v>
+        <v>187</v>
       </c>
       <c r="B7" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
       <c r="B8" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="B9" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="B10" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="B11" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="B12" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="B13" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="B14" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="B15" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="B16" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>162</v>
+        <v>197</v>
       </c>
       <c r="B17" s="10" t="b">
         <v>1</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>163</v>
+        <v>198</v>
       </c>
       <c r="B18" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>164</v>
+        <v>199</v>
       </c>
       <c r="B19" s="10">
         <v>20.0</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>166</v>
+        <v>201</v>
       </c>
       <c r="B20" s="10">
         <v>20.0</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>167</v>
+        <v>202</v>
       </c>
       <c r="B21" s="10">
         <v>5.0</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>168</v>
+        <v>203</v>
       </c>
       <c r="B22" s="10">
         <v>5.0</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>169</v>
+        <v>204</v>
       </c>
       <c r="B23" s="10">
         <v>1600.0</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>170</v>
+        <v>205</v>
       </c>
       <c r="B24" s="10">
         <v>0.85</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>171</v>
+        <v>206</v>
       </c>
       <c r="B25" s="10">
         <v>5.0</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>172</v>
+        <v>207</v>
       </c>
       <c r="B26" s="10">
         <v>1000.0</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>173</v>
+        <v>208</v>
       </c>
       <c r="B27" s="10">
         <v>300.0</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>174</v>
+        <v>209</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>175</v>
+        <v>210</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>176</v>
+        <v>211</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>178</v>
+        <v>213</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>179</v>
+        <v>214</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>180</v>
+        <v>215</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>181</v>
+        <v>216</v>
       </c>
       <c r="B32" s="10" t="b">
         <v>0</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>182</v>
+        <v>217</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>183</v>
+        <v>218</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>184</v>
+        <v>219</v>
       </c>
       <c r="B34" s="12"/>
       <c r="C34" s="10" t="s">
-        <v>165</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2607,7 +3202,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="B1" s="13">
         <v>46151.165393194446</v>
@@ -2634,15 +3229,15 @@
         <v>15</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>186</v>
+        <v>221</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>188</v>
+        <v>223</v>
       </c>
       <c r="B2" s="13">
         <v>46180.10313505787</v>
@@ -2672,12 +3267,12 @@
       <c r="L2" s="14"/>
       <c r="M2" s="10"/>
       <c r="Q2" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="B3" s="13">
         <v>46180.10315137732</v>
@@ -2702,12 +3297,12 @@
       </c>
       <c r="K3" s="10"/>
       <c r="Q3" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>190</v>
+        <v>225</v>
       </c>
       <c r="B4" s="13">
         <v>46180.103169236114</v>
@@ -2735,12 +3330,12 @@
       </c>
       <c r="K4" s="10"/>
       <c r="Q4" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>191</v>
+        <v>226</v>
       </c>
       <c r="B5" s="13">
         <v>46180.10318601852</v>
@@ -2768,12 +3363,12 @@
       </c>
       <c r="K5" s="10"/>
       <c r="Q5" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>192</v>
+        <v>227</v>
       </c>
       <c r="B6" s="13">
         <v>46180.103206631946</v>
@@ -2801,12 +3396,12 @@
       </c>
       <c r="K6" s="10"/>
       <c r="Q6" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>193</v>
+        <v>228</v>
       </c>
       <c r="B7" s="13">
         <v>46180.10322395833</v>
@@ -2831,12 +3426,12 @@
       </c>
       <c r="K7" s="10"/>
       <c r="Q7" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>194</v>
+        <v>229</v>
       </c>
       <c r="B8" s="13">
         <v>46180.103242303245</v>
@@ -2859,12 +3454,12 @@
       </c>
       <c r="K8" s="10"/>
       <c r="Q8" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="B9" s="13">
         <v>46180.103259386575</v>
@@ -2889,12 +3484,12 @@
         <v>45</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="B10" s="13">
         <v>46180.103281620366</v>
@@ -2919,12 +3514,12 @@
         <v>49</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>197</v>
+        <v>232</v>
       </c>
       <c r="B11" s="13">
         <v>46180.10330618055</v>
@@ -2949,12 +3544,12 @@
         <v>53</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="B12" s="13">
         <v>46180.10332761574</v>
@@ -2979,12 +3574,12 @@
         <v>55</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>199</v>
+        <v>234</v>
       </c>
       <c r="B13" s="13">
         <v>46180.10334641204</v>
@@ -3012,12 +3607,12 @@
         <v>59</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="B14" s="13">
         <v>46180.103362615744</v>
@@ -3045,12 +3640,12 @@
         <v>63</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>201</v>
+        <v>236</v>
       </c>
       <c r="B15" s="13">
         <v>46180.10338010416</v>
@@ -3078,12 +3673,12 @@
         <v>65</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="B16" s="13">
         <v>46180.10339710648</v>
@@ -3111,12 +3706,12 @@
         <v>71</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="B17" s="13">
         <v>46180.10341520833</v>
@@ -3144,12 +3739,12 @@
         <v>75</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="B18" s="13">
         <v>46180.10343418982</v>
@@ -3174,12 +3769,12 @@
         <v>80</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="B19" s="13">
         <v>46180.10344982639</v>
@@ -3207,12 +3802,12 @@
         <v>82</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>206</v>
+        <v>241</v>
       </c>
       <c r="B20" s="13">
         <v>46180.103465231485</v>
@@ -3237,12 +3832,12 @@
         <v>84</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>207</v>
+        <v>242</v>
       </c>
       <c r="B21" s="13">
         <v>46180.103480879625</v>
@@ -3267,12 +3862,12 @@
         <v>87</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>208</v>
+        <v>243</v>
       </c>
       <c r="B22" s="13">
         <v>46180.103501053236</v>
@@ -3297,12 +3892,12 @@
         <v>90</v>
       </c>
       <c r="Q22" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>209</v>
+        <v>244</v>
       </c>
       <c r="B23" s="13">
         <v>46180.10351888889</v>
@@ -3330,12 +3925,12 @@
         <v>93</v>
       </c>
       <c r="Q23" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="s">
-        <v>210</v>
+        <v>245</v>
       </c>
       <c r="B24" s="13">
         <v>46180.103536608796</v>
@@ -3363,12 +3958,12 @@
         <v>98</v>
       </c>
       <c r="Q24" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="s">
-        <v>211</v>
+        <v>246</v>
       </c>
       <c r="B25" s="13">
         <v>46180.103555381946</v>
@@ -3393,12 +3988,12 @@
         <v>102</v>
       </c>
       <c r="Q25" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="s">
-        <v>212</v>
+        <v>247</v>
       </c>
       <c r="B26" s="13">
         <v>46180.10357407408</v>
@@ -3423,12 +4018,12 @@
         <v>104</v>
       </c>
       <c r="Q26" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="s">
-        <v>213</v>
+        <v>248</v>
       </c>
       <c r="B27" s="13">
         <v>46180.103594050925</v>
@@ -3453,12 +4048,12 @@
         <v>107</v>
       </c>
       <c r="Q27" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="s">
-        <v>214</v>
+        <v>249</v>
       </c>
       <c r="B28" s="13">
         <v>46180.10361086806</v>
@@ -3483,12 +4078,12 @@
         <v>110</v>
       </c>
       <c r="Q28" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="s">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="B29" s="13">
         <v>46180.10362674769</v>
@@ -3513,12 +4108,12 @@
         <v>113</v>
       </c>
       <c r="Q29" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="s">
-        <v>216</v>
+        <v>251</v>
       </c>
       <c r="B30" s="13">
         <v>46180.10364325231</v>
@@ -3544,12 +4139,12 @@
         <v>115</v>
       </c>
       <c r="Q30" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="s">
-        <v>217</v>
+        <v>252</v>
       </c>
       <c r="B31" s="13">
         <v>46180.10365928241</v>
@@ -3574,12 +4169,12 @@
         <v>118</v>
       </c>
       <c r="Q31" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="B32" s="13">
         <v>46180.10367861111</v>
@@ -3601,12 +4196,12 @@
         <v>121</v>
       </c>
       <c r="Q32" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="B33" s="13">
         <v>46180.103699074076</v>
@@ -3631,12 +4226,12 @@
         <v>123</v>
       </c>
       <c r="Q33" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
       <c r="B34" s="13">
         <v>46180.11010986111</v>
@@ -3663,12 +4258,12 @@
         <v>126</v>
       </c>
       <c r="Q34" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="B35" s="13">
         <v>46180.11529725694</v>
@@ -3695,12 +4290,12 @@
         <v>128</v>
       </c>
       <c r="Q35" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="s">
-        <v>222</v>
+        <v>257</v>
       </c>
       <c r="B36" s="13">
         <v>46180.1201821412</v>
@@ -3727,12 +4322,12 @@
         <v>130</v>
       </c>
       <c r="Q36" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
       <c r="B37" s="13">
         <v>46180.12604854167</v>
@@ -3759,12 +4354,12 @@
         <v>133</v>
       </c>
       <c r="Q37" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="B38" s="13">
         <v>46180.133690347226</v>
@@ -3791,7 +4386,550 @@
         <v>135</v>
       </c>
       <c r="Q38" s="10" t="s">
-        <v>187</v>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="B39" s="13">
+        <v>46180.14498915509</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="J39" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q39" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="B40" s="13">
+        <v>46180.42403625</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J40" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q40" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="B41" s="13">
+        <v>46180.42562646991</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="J41" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="Q41" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="B42" s="13">
+        <v>46180.42677348379</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="J42" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q42" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="B43" s="13">
+        <v>46180.42843393519</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="J43" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q43" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="s">
+        <v>265</v>
+      </c>
+      <c r="B44" s="13">
+        <v>46180.43111269676</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="J44" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q44" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="B45" s="13">
+        <v>46180.48142487268</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="J45" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q45" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="B46" s="13">
+        <v>46180.49306246528</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I46" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J46" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q46" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="B47" s="13">
+        <v>46180.49664386574</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="J47" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q47" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="B48" s="13">
+        <v>46180.49833422454</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J48" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q48" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B49" s="13">
+        <v>46180.5560616088</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J49" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q49" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="B50" s="13">
+        <v>46180.556612025466</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J50" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q50" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="B51" s="13">
+        <v>46180.55723766204</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J51" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q51" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="B52" s="13">
+        <v>46180.55785491898</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H52" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J52" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q52" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B53" s="13">
+        <v>46180.55835274306</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J53" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q53" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="B54" s="13">
+        <v>46180.5592303125</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J54" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q54" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="B55" s="13">
+        <v>46180.55976952546</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H55" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J55" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q55" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="B56" s="13">
+        <v>46180.56037356482</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H56" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J56" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q56" s="10" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -3808,8 +4946,15 @@
     <hyperlink r:id="rId10" ref="I33"/>
     <hyperlink r:id="rId11" ref="I36"/>
     <hyperlink r:id="rId12" ref="I37"/>
+    <hyperlink r:id="rId13" ref="I41"/>
+    <hyperlink r:id="rId14" ref="I42"/>
+    <hyperlink r:id="rId15" ref="I43"/>
+    <hyperlink r:id="rId16" ref="I44"/>
+    <hyperlink r:id="rId17" ref="I45"/>
+    <hyperlink r:id="rId18" ref="I46"/>
+    <hyperlink r:id="rId19" ref="I47"/>
   </hyperlinks>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId20"/>
 </worksheet>
 </file>
 
@@ -3845,69 +4990,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>225</v>
+        <v>278</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>226</v>
+        <v>279</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>227</v>
+        <v>280</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>228</v>
+        <v>281</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>229</v>
+        <v>282</v>
       </c>
       <c r="G1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>230</v>
+        <v>283</v>
       </c>
       <c r="I1" s="15" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>231</v>
+        <v>284</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>232</v>
+        <v>285</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>233</v>
+        <v>286</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>234</v>
+        <v>287</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>235</v>
+        <v>288</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>236</v>
+        <v>289</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>237</v>
+        <v>290</v>
       </c>
       <c r="Q1" s="15" t="s">
-        <v>238</v>
+        <v>291</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>239</v>
+        <v>292</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>240</v>
+        <v>293</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>241</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="B2" s="13">
         <v>46151.16717461805</v>
@@ -3936,7 +5081,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>242</v>
+        <v>295</v>
       </c>
       <c r="O2" s="13">
         <v>46173.25955616898</v>
@@ -3946,7 +5091,7 @@
       </c>
       <c r="S2" s="14"/>
       <c r="T2" s="10" t="s">
-        <v>243</v>
+        <v>296</v>
       </c>
       <c r="U2" s="10"/>
       <c r="V2" s="10"/>
@@ -12071,7 +13216,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>230</v>
+        <v>283</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>5</v>
@@ -12080,7 +13225,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>235</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2">
@@ -12091,13 +13236,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>244</v>
+        <v>297</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>245</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3">
@@ -12114,7 +13259,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>246</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4">
@@ -12131,12 +13276,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>242</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="s">
-        <v>247</v>
+        <v>300</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>54</v>
@@ -12148,7 +13293,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>248</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6">
@@ -12180,12 +13325,12 @@
         <v>16</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>249</v>
+        <v>302</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="s">
-        <v>250</v>
+        <v>303</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>132</v>
@@ -12193,12 +13338,12 @@
     </row>
     <row r="11">
       <c r="B11" s="17" t="s">
-        <v>251</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="s">
-        <v>252</v>
+        <v>304</v>
       </c>
     </row>
     <row r="13">
@@ -12208,17 +13353,17 @@
     </row>
     <row r="14">
       <c r="B14" s="17" t="s">
-        <v>253</v>
+        <v>305</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="s">
-        <v>254</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="s">
-        <v>255</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17">
@@ -12228,12 +13373,12 @@
     </row>
     <row r="18">
       <c r="B18" s="17" t="s">
-        <v>256</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="s">
-        <v>257</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20">
@@ -12248,7 +13393,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="17" t="s">
-        <v>258</v>
+        <v>309</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -12258,7 +13403,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="17" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v16 2026-06-22 02:29 IST [3x-daily]
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="408">
   <si>
     <t>Timestamp</t>
   </si>
@@ -707,6 +707,45 @@
     <t>https://drive.google.com/open?id=1YvGUet-8ZHxt1jFQR8I_gPQdc1doWqR5</t>
   </si>
   <si>
+    <t xml:space="preserve">Prakash Yelwande </t>
+  </si>
+  <si>
+    <t>A1101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pegion dropping, looks worst from our kitchen exactly opposite to kitchen of A1101,the wall in duct </t>
+  </si>
+  <si>
+    <t>Pegion dropping, looks worst from our kitchen exactly opposite to kitchen of A1101,the wall in duct, kindly repaint without  fail as we will need to see it life long and apply pegion nets at the earliest to avoid this</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1n-oao6jmKAmA52WIk9PbmJ3ABMLn9v05</t>
+  </si>
+  <si>
+    <t>A wing entrance from road side is fully leaking and is visible during rains, kindly check and correct the leakage in cracks</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1d6HTd7pAx77_0Tp6fFw1klWmAZnBpp0o</t>
+  </si>
+  <si>
+    <t>Dadasaheb Salunke</t>
+  </si>
+  <si>
+    <t>B-901</t>
+  </si>
+  <si>
+    <t>With reference to the attached image, the passage area behind the B-Wing lift lobby is currently being used for two-wheeler parking. Several plumbing pipes are installed along the wall in this area, and there is a high risk of damage to these pipes due to contact from front tyres of parked two-wheelers, particularly from tyres and vehicle movement.  It is recommended to either:  1. Prohibit two-wheeler parking in this passage area, or 2. Protect the plumbing pipes by installing a suitable steel safety grid/guard along the wall.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1wsXPPHRxXbLq7x-0TouQPurwA60hwLh_</t>
+  </si>
+  <si>
+    <t>Dadasaheb S</t>
+  </si>
+  <si>
+    <t>Some basic lift settings appear to be missing or need adjustment:  1. Double-tap to cancel a floor call is not working.  2. The touch buttons are overly sensitive; even slight body contact can trigger multiple floor selections.  3. Not sure if the occupancy sensor is enabled. The cabin lights and fan should turn off when the lift is unoccupied. Currently, the fan can be heard running from outside even when the lift is empty.</t>
+  </si>
+  <si>
     <t>Key</t>
   </si>
   <si>
@@ -1095,6 +1134,18 @@
   </si>
   <si>
     <t>TKT-00076</t>
+  </si>
+  <si>
+    <t>TKT-00077</t>
+  </si>
+  <si>
+    <t>TKT-00078</t>
+  </si>
+  <si>
+    <t>TKT-00079</t>
+  </si>
+  <si>
+    <t>TKT-00080</t>
   </si>
   <si>
     <t>Ticket ID</t>
@@ -1431,7 +1482,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I77" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I81" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="9">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Resident Name" id="2"/>
@@ -3456,6 +3507,107 @@
         <v>227</v>
       </c>
     </row>
+    <row r="78" ht="22.5" customHeight="1">
+      <c r="A78" s="6">
+        <v>46190.50344489583</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H78" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="79" ht="22.5" customHeight="1">
+      <c r="A79" s="6">
+        <v>46190.532821886576</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="I79" s="8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="80" ht="22.5" customHeight="1">
+      <c r="A80" s="6">
+        <v>46193.184405567124</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H80" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="I80" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="81" ht="22.5" customHeight="1">
+      <c r="A81" s="6">
+        <v>46193.18515243055</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>240</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="I15"/>
@@ -3483,10 +3635,13 @@
     <hyperlink r:id="rId23" ref="I73"/>
     <hyperlink r:id="rId24" ref="I76"/>
     <hyperlink r:id="rId25" ref="I77"/>
+    <hyperlink r:id="rId26" ref="I78"/>
+    <hyperlink r:id="rId27" ref="I79"/>
+    <hyperlink r:id="rId28" ref="I80"/>
   </hyperlinks>
-  <drawing r:id="rId26"/>
+  <drawing r:id="rId29"/>
   <tableParts count="1">
-    <tablePart r:id="rId28"/>
+    <tablePart r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3505,382 +3660,382 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="B6" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="B7" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="B8" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="B9" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="B10" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="B11" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="B12" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="B13" s="11" t="b">
         <v>0</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="B14" s="11" t="b">
         <v>0</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="B15" s="11" t="b">
         <v>0</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="B16" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="B17" s="11" t="b">
         <v>1</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="B18" s="11" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="B19" s="11">
         <v>20.0</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="B20" s="11">
         <v>20.0</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="B21" s="11">
         <v>5.0</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="B22" s="11">
         <v>5.0</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="B23" s="11">
         <v>1600.0</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="B24" s="11">
         <v>0.85</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="B25" s="11">
         <v>5.0</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="B26" s="11">
         <v>1000.0</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
       <c r="B27" s="11">
         <v>300.0</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>269</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="B31" s="13"/>
       <c r="C31" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
       <c r="B32" s="11" t="b">
         <v>0</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -3906,7 +4061,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="B1" s="15">
         <v>46151.165393194446</v>
@@ -3933,15 +4088,15 @@
         <v>15</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="B2" s="15">
         <v>46180.10313505787</v>
@@ -3971,12 +4126,12 @@
       <c r="L2" s="16"/>
       <c r="M2" s="11"/>
       <c r="Q2" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="B3" s="15">
         <v>46180.10315137732</v>
@@ -4001,12 +4156,12 @@
       </c>
       <c r="K3" s="11"/>
       <c r="Q3" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="B4" s="15">
         <v>46180.103169236114</v>
@@ -4034,12 +4189,12 @@
       </c>
       <c r="K4" s="11"/>
       <c r="Q4" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="B5" s="15">
         <v>46180.10318601852</v>
@@ -4067,12 +4222,12 @@
       </c>
       <c r="K5" s="11"/>
       <c r="Q5" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="B6" s="15">
         <v>46180.103206631946</v>
@@ -4100,12 +4255,12 @@
       </c>
       <c r="K6" s="11"/>
       <c r="Q6" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="B7" s="15">
         <v>46180.10322395833</v>
@@ -4130,12 +4285,12 @@
       </c>
       <c r="K7" s="11"/>
       <c r="Q7" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="B8" s="15">
         <v>46180.103242303245</v>
@@ -4158,12 +4313,12 @@
       </c>
       <c r="K8" s="11"/>
       <c r="Q8" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="B9" s="15">
         <v>46180.103259386575</v>
@@ -4188,12 +4343,12 @@
         <v>45</v>
       </c>
       <c r="Q9" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
       <c r="B10" s="15">
         <v>46180.103281620366</v>
@@ -4218,12 +4373,12 @@
         <v>49</v>
       </c>
       <c r="Q10" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="B11" s="15">
         <v>46180.10330618055</v>
@@ -4248,12 +4403,12 @@
         <v>53</v>
       </c>
       <c r="Q11" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
       <c r="B12" s="15">
         <v>46180.10332761574</v>
@@ -4278,12 +4433,12 @@
         <v>55</v>
       </c>
       <c r="Q12" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="B13" s="15">
         <v>46180.10334641204</v>
@@ -4311,12 +4466,12 @@
         <v>59</v>
       </c>
       <c r="Q13" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="B14" s="15">
         <v>46180.103362615744</v>
@@ -4344,12 +4499,12 @@
         <v>63</v>
       </c>
       <c r="Q14" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
       <c r="B15" s="15">
         <v>46180.10338010416</v>
@@ -4377,12 +4532,12 @@
         <v>65</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="B16" s="15">
         <v>46180.10339710648</v>
@@ -4410,12 +4565,12 @@
         <v>71</v>
       </c>
       <c r="Q16" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="B17" s="15">
         <v>46180.10341520833</v>
@@ -4443,12 +4598,12 @@
         <v>75</v>
       </c>
       <c r="Q17" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="B18" s="15">
         <v>46180.10343418982</v>
@@ -4473,12 +4628,12 @@
         <v>80</v>
       </c>
       <c r="Q18" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="B19" s="15">
         <v>46180.10344982639</v>
@@ -4506,12 +4661,12 @@
         <v>82</v>
       </c>
       <c r="Q19" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="B20" s="15">
         <v>46180.103465231485</v>
@@ -4536,12 +4691,12 @@
         <v>84</v>
       </c>
       <c r="Q20" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="B21" s="15">
         <v>46180.103480879625</v>
@@ -4566,12 +4721,12 @@
         <v>87</v>
       </c>
       <c r="Q21" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="B22" s="15">
         <v>46180.103501053236</v>
@@ -4596,12 +4751,12 @@
         <v>90</v>
       </c>
       <c r="Q22" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="B23" s="15">
         <v>46180.10351888889</v>
@@ -4629,12 +4784,12 @@
         <v>93</v>
       </c>
       <c r="Q23" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="B24" s="15">
         <v>46180.103536608796</v>
@@ -4662,12 +4817,12 @@
         <v>98</v>
       </c>
       <c r="Q24" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="B25" s="15">
         <v>46180.103555381946</v>
@@ -4692,12 +4847,12 @@
         <v>102</v>
       </c>
       <c r="Q25" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="B26" s="15">
         <v>46180.10357407408</v>
@@ -4722,12 +4877,12 @@
         <v>104</v>
       </c>
       <c r="Q26" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="B27" s="15">
         <v>46180.103594050925</v>
@@ -4752,12 +4907,12 @@
         <v>107</v>
       </c>
       <c r="Q27" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
       <c r="B28" s="15">
         <v>46180.10361086806</v>
@@ -4782,12 +4937,12 @@
         <v>110</v>
       </c>
       <c r="Q28" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
       <c r="B29" s="15">
         <v>46180.10362674769</v>
@@ -4812,12 +4967,12 @@
         <v>113</v>
       </c>
       <c r="Q29" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="B30" s="15">
         <v>46180.10364325231</v>
@@ -4843,12 +4998,12 @@
         <v>115</v>
       </c>
       <c r="Q30" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
       <c r="B31" s="15">
         <v>46180.10365928241</v>
@@ -4873,12 +5028,12 @@
         <v>118</v>
       </c>
       <c r="Q31" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="B32" s="15">
         <v>46180.10367861111</v>
@@ -4900,12 +5055,12 @@
         <v>121</v>
       </c>
       <c r="Q32" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="B33" s="15">
         <v>46180.103699074076</v>
@@ -4930,12 +5085,12 @@
         <v>123</v>
       </c>
       <c r="Q33" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="B34" s="15">
         <v>46180.11010986111</v>
@@ -4962,12 +5117,12 @@
         <v>126</v>
       </c>
       <c r="Q34" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="B35" s="15">
         <v>46180.11529725694</v>
@@ -4994,12 +5149,12 @@
         <v>128</v>
       </c>
       <c r="Q35" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="B36" s="15">
         <v>46180.1201821412</v>
@@ -5026,12 +5181,12 @@
         <v>130</v>
       </c>
       <c r="Q36" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="B37" s="15">
         <v>46180.12604854167</v>
@@ -5058,12 +5213,12 @@
         <v>133</v>
       </c>
       <c r="Q37" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="B38" s="15">
         <v>46180.133690347226</v>
@@ -5090,12 +5245,12 @@
         <v>135</v>
       </c>
       <c r="Q38" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="B39" s="15">
         <v>46180.14498915509</v>
@@ -5119,12 +5274,12 @@
         <v>137</v>
       </c>
       <c r="Q39" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="B40" s="15">
         <v>46180.42403625</v>
@@ -5148,12 +5303,12 @@
         <v>140</v>
       </c>
       <c r="Q40" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="B41" s="15">
         <v>46180.42562646991</v>
@@ -5177,12 +5332,12 @@
         <v>142</v>
       </c>
       <c r="Q41" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="B42" s="15">
         <v>46180.42677348379</v>
@@ -5206,12 +5361,12 @@
         <v>144</v>
       </c>
       <c r="Q42" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="B43" s="15">
         <v>46180.42843393519</v>
@@ -5235,12 +5390,12 @@
         <v>146</v>
       </c>
       <c r="Q43" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="B44" s="15">
         <v>46180.43111269676</v>
@@ -5264,12 +5419,12 @@
         <v>148</v>
       </c>
       <c r="Q44" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="B45" s="15">
         <v>46180.48142487268</v>
@@ -5293,12 +5448,12 @@
         <v>150</v>
       </c>
       <c r="Q45" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="B46" s="15">
         <v>46180.49306246528</v>
@@ -5322,12 +5477,12 @@
         <v>153</v>
       </c>
       <c r="Q46" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="B47" s="15">
         <v>46180.49664386574</v>
@@ -5351,12 +5506,12 @@
         <v>155</v>
       </c>
       <c r="Q47" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="B48" s="15">
         <v>46180.49833422454</v>
@@ -5377,12 +5532,12 @@
         <v>158</v>
       </c>
       <c r="Q48" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="B49" s="15">
         <v>46180.5560616088</v>
@@ -5403,12 +5558,12 @@
         <v>160</v>
       </c>
       <c r="Q49" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="B50" s="15">
         <v>46180.556612025466</v>
@@ -5429,12 +5584,12 @@
         <v>161</v>
       </c>
       <c r="Q50" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="B51" s="15">
         <v>46180.55723766204</v>
@@ -5455,12 +5610,12 @@
         <v>163</v>
       </c>
       <c r="Q51" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="B52" s="15">
         <v>46180.55785491898</v>
@@ -5481,12 +5636,12 @@
         <v>165</v>
       </c>
       <c r="Q52" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="B53" s="15">
         <v>46180.55835274306</v>
@@ -5507,12 +5662,12 @@
         <v>166</v>
       </c>
       <c r="Q53" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="B54" s="15">
         <v>46180.5592303125</v>
@@ -5533,12 +5688,12 @@
         <v>168</v>
       </c>
       <c r="Q54" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="B55" s="15">
         <v>46180.55976952546</v>
@@ -5559,12 +5714,12 @@
         <v>170</v>
       </c>
       <c r="Q55" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="B56" s="15">
         <v>46180.56037356482</v>
@@ -5585,12 +5740,12 @@
         <v>172</v>
       </c>
       <c r="Q56" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="B57" s="15">
         <v>46180.841951689814</v>
@@ -5617,12 +5772,12 @@
         <v>175</v>
       </c>
       <c r="Q57" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="B58" s="15">
         <v>46180.849617430555</v>
@@ -5649,12 +5804,12 @@
         <v>178</v>
       </c>
       <c r="Q58" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="B59" s="15">
         <v>46180.89295709491</v>
@@ -5678,12 +5833,12 @@
         <v>183</v>
       </c>
       <c r="Q59" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="B60" s="15">
         <v>46180.906154386576</v>
@@ -5710,12 +5865,12 @@
         <v>184</v>
       </c>
       <c r="Q60" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="B61" s="15">
         <v>46180.91151877315</v>
@@ -5742,12 +5897,12 @@
         <v>186</v>
       </c>
       <c r="Q61" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="B62" s="15">
         <v>46180.9191175</v>
@@ -5774,12 +5929,12 @@
         <v>188</v>
       </c>
       <c r="Q62" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="B63" s="15">
         <v>46180.92425851852</v>
@@ -5806,12 +5961,12 @@
         <v>191</v>
       </c>
       <c r="Q63" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="B64" s="15">
         <v>46180.944133819445</v>
@@ -5835,12 +5990,12 @@
         <v>195</v>
       </c>
       <c r="Q64" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="B65" s="15">
         <v>46181.34467190973</v>
@@ -5864,12 +6019,12 @@
         <v>199</v>
       </c>
       <c r="Q65" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="B66" s="15">
         <v>46181.39693835648</v>
@@ -5893,12 +6048,12 @@
         <v>201</v>
       </c>
       <c r="Q66" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="B67" s="15">
         <v>46181.966292604164</v>
@@ -5925,12 +6080,12 @@
         <v>204</v>
       </c>
       <c r="Q67" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
       <c r="B68" s="15">
         <v>46183.84682266203</v>
@@ -5954,12 +6109,12 @@
         <v>206</v>
       </c>
       <c r="Q68" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="B69" s="15">
         <v>46183.8483637037</v>
@@ -5983,12 +6138,12 @@
         <v>209</v>
       </c>
       <c r="Q69" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="11" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
       <c r="B70" s="15">
         <v>46183.84967077547</v>
@@ -6009,12 +6164,12 @@
         <v>211</v>
       </c>
       <c r="Q70" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="B71" s="15">
         <v>46183.85057898148</v>
@@ -6038,12 +6193,12 @@
         <v>212</v>
       </c>
       <c r="Q71" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="11" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="B72" s="15">
         <v>46183.85173738426</v>
@@ -6067,12 +6222,12 @@
         <v>214</v>
       </c>
       <c r="Q72" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="11" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="B73" s="15">
         <v>46183.85328108796</v>
@@ -6096,12 +6251,12 @@
         <v>217</v>
       </c>
       <c r="Q73" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="11" t="s">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="B74" s="15">
         <v>46183.85490774305</v>
@@ -6125,12 +6280,12 @@
         <v>220</v>
       </c>
       <c r="Q74" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="11" t="s">
-        <v>356</v>
+        <v>369</v>
       </c>
       <c r="B75" s="15">
         <v>46183.856149907406</v>
@@ -6154,12 +6309,12 @@
         <v>223</v>
       </c>
       <c r="Q75" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="11" t="s">
-        <v>357</v>
+        <v>370</v>
       </c>
       <c r="B76" s="15">
         <v>46185.945908333335</v>
@@ -6183,7 +6338,132 @@
         <v>226</v>
       </c>
       <c r="Q76" s="11" t="s">
-        <v>282</v>
+        <v>295</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="B77" s="15">
+        <v>46190.503476666665</v>
+      </c>
+      <c r="C77" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="D77" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I77" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="J77" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q77" s="11" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="B78" s="15">
+        <v>46190.53284886574</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="D78" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="F78" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H78" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I78" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="J78" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q78" s="11" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="B79" s="15">
+        <v>46193.18443314815</v>
+      </c>
+      <c r="C79" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D79" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="E79" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F79" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H79" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="I79" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="J79" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q79" s="11" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="s">
+        <v>374</v>
+      </c>
+      <c r="B80" s="15">
+        <v>46193.18517116898</v>
+      </c>
+      <c r="C80" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="D80" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="E80" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F80" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H80" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J80" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q80" s="11" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -6213,8 +6493,11 @@
     <hyperlink r:id="rId23" ref="I72"/>
     <hyperlink r:id="rId24" ref="I75"/>
     <hyperlink r:id="rId25" ref="I76"/>
+    <hyperlink r:id="rId26" ref="I77"/>
+    <hyperlink r:id="rId27" ref="I78"/>
+    <hyperlink r:id="rId28" ref="I79"/>
   </hyperlinks>
-  <drawing r:id="rId26"/>
+  <drawing r:id="rId29"/>
 </worksheet>
 </file>
 
@@ -6250,69 +6533,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="18" t="s">
-        <v>358</v>
+        <v>375</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>359</v>
+        <v>376</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>360</v>
+        <v>377</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>361</v>
+        <v>378</v>
       </c>
       <c r="E1" s="18" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>362</v>
+        <v>379</v>
       </c>
       <c r="G1" s="18" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>363</v>
+        <v>380</v>
       </c>
       <c r="I1" s="18" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="18" t="s">
-        <v>364</v>
+        <v>381</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>365</v>
+        <v>382</v>
       </c>
       <c r="L1" s="18" t="s">
-        <v>366</v>
+        <v>383</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>367</v>
+        <v>384</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>368</v>
+        <v>385</v>
       </c>
       <c r="O1" s="18" t="s">
-        <v>369</v>
+        <v>386</v>
       </c>
       <c r="P1" s="18" t="s">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="Q1" s="18" t="s">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="R1" s="18" t="s">
-        <v>372</v>
+        <v>389</v>
       </c>
       <c r="S1" s="18" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="T1" s="18" t="s">
-        <v>374</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="B2" s="15">
         <v>46151.16717461805</v>
@@ -6341,7 +6624,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>375</v>
+        <v>392</v>
       </c>
       <c r="O2" s="15">
         <v>46173.25955616898</v>
@@ -6351,7 +6634,7 @@
       </c>
       <c r="S2" s="16"/>
       <c r="T2" s="11" t="s">
-        <v>376</v>
+        <v>393</v>
       </c>
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
@@ -14476,7 +14759,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>363</v>
+        <v>380</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>5</v>
@@ -14485,7 +14768,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>368</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2">
@@ -14496,13 +14779,13 @@
         <v>58</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>377</v>
+        <v>394</v>
       </c>
       <c r="D2" s="20" t="s">
         <v>34</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>378</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3">
@@ -14519,7 +14802,7 @@
         <v>14</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>379</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4">
@@ -14536,12 +14819,12 @@
         <v>44</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>375</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="s">
-        <v>380</v>
+        <v>397</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>54</v>
@@ -14553,7 +14836,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>381</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6">
@@ -14585,12 +14868,12 @@
         <v>16</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>382</v>
+        <v>399</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="s">
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>132</v>
@@ -14603,7 +14886,7 @@
     </row>
     <row r="12">
       <c r="B12" s="20" t="s">
-        <v>384</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13">
@@ -14613,7 +14896,7 @@
     </row>
     <row r="14">
       <c r="B14" s="20" t="s">
-        <v>385</v>
+        <v>402</v>
       </c>
     </row>
     <row r="15">
@@ -14623,7 +14906,7 @@
     </row>
     <row r="16">
       <c r="B16" s="20" t="s">
-        <v>386</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17">
@@ -14633,12 +14916,12 @@
     </row>
     <row r="18">
       <c r="B18" s="20" t="s">
-        <v>387</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="20" t="s">
-        <v>388</v>
+        <v>405</v>
       </c>
     </row>
     <row r="20">
@@ -14653,7 +14936,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="20" t="s">
-        <v>389</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -14663,7 +14946,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="20" t="s">
-        <v>390</v>
+        <v>407</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
backup: v21 2026-07-06 02:29 IST [3x-daily]
</commit_message>
<xml_diff>
--- a/backups/ta-issue-manager.xlsx
+++ b/backups/ta-issue-manager.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1929" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2016" uniqueCount="561">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1704,147 +1704,84 @@
     <t>TKT-00083</t>
   </si>
   <si>
-    <t>51. Below pool area paint patches (under one)</t>
-  </si>
-  <si>
     <t>TKT-00084</t>
   </si>
   <si>
-    <t>52. Gym Area – Cracks on the wall, plaster/paint/electric supply, flooring</t>
-  </si>
-  <si>
     <t>TKT-00085</t>
   </si>
   <si>
-    <t>53. Open Electrical points near gym area possible for lights as depicted by</t>
-  </si>
-  <si>
     <t>TKT-00086</t>
   </si>
   <si>
-    <t>54. STP Operation Room – Working/Finishing</t>
-  </si>
-  <si>
     <t>TKT-00087</t>
   </si>
   <si>
-    <t>56. A Wing Service lift marble crack change required</t>
-  </si>
-  <si>
     <t>TKT-00088</t>
   </si>
   <si>
-    <t>57. Security Gate 2: Cabin</t>
-  </si>
-  <si>
     <t>TKT-00089</t>
   </si>
   <si>
-    <t>58. A Building Fire Door Handle missing</t>
-  </si>
-  <si>
     <t>TKT-00090</t>
   </si>
   <si>
-    <t>59. Transformer Operational and to be locked</t>
-  </si>
-  <si>
     <t>TKT-00091</t>
   </si>
   <si>
-    <t>60. A Wing Gate 1st floor access to pool area</t>
-  </si>
-  <si>
     <t>TKT-00092</t>
   </si>
   <si>
-    <t>61. Steel Railing Too</t>
-  </si>
-  <si>
     <t>TKT-00093</t>
   </si>
   <si>
-    <t>62. Electrical points Terrace (A)</t>
-  </si>
-  <si>
     <t>TKT-00094</t>
   </si>
   <si>
-    <t>63. Supporter gas O cap broken</t>
-  </si>
-  <si>
     <t>TKT-00095</t>
   </si>
   <si>
-    <t>64. Pump cover fire fighting cover</t>
-  </si>
-  <si>
     <t>TKT-00096</t>
   </si>
   <si>
-    <t>65. Water levelling B wing above 3 series</t>
-  </si>
-  <si>
     <t>TKT-00097</t>
   </si>
   <si>
-    <t>66. Water flow terrace</t>
-  </si>
-  <si>
     <t>TKT-00098</t>
   </si>
   <si>
-    <t>67. AC duct placement B problem</t>
+    <t>https://drive.google.com/file/d/10Q9xD34OOrMaTzB5o_wKm2cPpluO9IhS/view?usp=drive_link, https://drive.google.com/file/d/1ljpeEbQtAkhE8_HCpbz_N13yWG_Vcbzq/view?usp=drive_link, https://drive.google.com/file/d/1u-T8R05GIcKX11AiwK54hqkg9O363TIC/view?usp=drive_link</t>
   </si>
   <si>
     <t>TKT-00099</t>
   </si>
   <si>
-    <t>68. Wire mesh safety C wing</t>
-  </si>
-  <si>
     <t>TKT-00100</t>
   </si>
   <si>
-    <t>69. Club House Toilet flush – Toilet (1) choked</t>
-  </si>
-  <si>
     <t>TKT-00101</t>
   </si>
   <si>
-    <t>70. Water level terrace C tower</t>
-  </si>
-  <si>
     <t>TKT-00102</t>
   </si>
   <si>
-    <t>71. Water seepage – Plumbing tank leaky</t>
+    <t>https://drive.google.com/file/d/1SeK5PE9OHSqfhwpmz44ApedHHzWNpy2_/view?usp=drive_link, https://drive.google.com/file/d/1ep6Ezj3vuLtHwEqpjUywNgLHYk3bgETQ/view?usp=drive_link</t>
   </si>
   <si>
     <t>TKT-00103</t>
   </si>
   <si>
-    <t>72. Hanging plumbing pipe</t>
-  </si>
-  <si>
     <t>TKT-00104</t>
   </si>
   <si>
-    <t>73. Air pipe WC pipe extend heights</t>
-  </si>
-  <si>
     <t>TKT-00105</t>
   </si>
   <si>
-    <t>74. Tile Broken (C)</t>
+    <t>https://drive.google.com/file/d/16rWrbxbJpHXroJ6I6z81X-yq0q7v4BhP/view?usp=drive_link, https://drive.google.com/file/d/1caWLT5wGxEMDIneGMd1sy8BWAvHy1BOJ/view?usp=drive_link, https://drive.google.com/file/d/1Xzl5XeoGwQxzw5uQnIumiwHQbyEERoFq/view?usp=drive_link</t>
   </si>
   <si>
     <t>TKT-00106</t>
   </si>
   <si>
-    <t>75. C Wing B U Cup</t>
-  </si>
-  <si>
     <t>TKT-00107</t>
   </si>
   <si>
@@ -1900,6 +1837,42 @@
   </si>
   <si>
     <t>TKT-00125</t>
+  </si>
+  <si>
+    <t>TKT-00126</t>
+  </si>
+  <si>
+    <t>TKT-00127</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1NzNLE1JgB8RgETpeR0aiBR-qh7OExJ9G/view?usp=drive_link, https://drive.google.com/file/d/1QMAMdMFeB3z0LRct6H_z3FM3QMXMt1bx/view?usp=drive_link, https://drive.google.com/file/d/1dZGsgwopKQXjyV-bH8ab7MGNX_f887yS/view?usp=drive_link, https://drive.google.com/file/d/10g2PlLu6frzgBFzBpb1BO9uchGA-1d6A/view?usp=drive_link, https://drive.google.com/file/d/1SlpqYq5lwcl3Vj1TX3hSiFcEQJNCyiID/view?usp=drive_link, https://drive.google.com/file/d/17iz9gfmaI469op4Tr8DL4pRYI-fkvQpJ/view?usp=drive_link,  https://drive.google.com/file/d/1GFw-oQ3u34EOtHw16_ByB4BPMNqwz6oj/view?usp=drive_link, https://drive.google.com/file/d/1X-QrW0wHDuKYyenvozxJKXO3JTDs4qBc/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>TKT-00128</t>
+  </si>
+  <si>
+    <t>TKT-00129</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/194fbZXRmuM8lsHLJClTIwUgkfIkmRGT8/view?usp=drive_link, https://drive.google.com/file/d/1LvWcTZMv96DrbhlExi04ULjUacHNKVt8/view?usp=drive_link, https://drive.google.com/file/d/10VVUINLggdthS2o-800Pf1ZYn9Fs7F2D/view?usp=drive_link, https://drive.google.com/file/d/1a-xc_cxDGl_wSLMheHENGOW_QouqEb8J/view?usp=drive_link, https://drive.google.com/file/d/1g4QaRlwxikDOJ9xR2ylSpGlNV3nE7939/view?usp=drive_link, https://drive.google.com/file/d/1d96VV3hA6xfEsbvdpu6aGQoMHQpPj2dr/view?usp=drive_link, https://drive.google.com/file/d/15_HB24ekNMuEOqu_16jtCMTXXGdtQ9bj/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>TKT-00130</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1_8mips4jlqLm6_jRwDRJW0RRiq-sClyS/view?usp=drive_link, https://drive.google.com/file/d/1qYr4AvLDRuemFzPtyah6ej4h99qKCMxk/view?usp=drive_link, https://drive.google.com/file/d/135DAIwsBFEVnPWEGcuxDJxgOnGAQJwDw/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>TKT-00131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://drive.google.com/file/d/1kJ3ZHARMsVJkaN4vJ0nCpLZ2E-8Tp8hQ/view?usp=drive_link, https://drive.google.com/file/d/1hTTaq4-hoNoWwCTHA0HjpAiZ2JB4S5Zl/view?usp=drive_link, </t>
+  </si>
+  <si>
+    <t>TKT-00132</t>
+  </si>
+  <si>
+    <t>TKT-00133</t>
   </si>
   <si>
     <t>Ticket ID</t>
@@ -8869,8 +8842,11 @@
       <c r="H83" s="24" t="s">
         <v>17</v>
       </c>
+      <c r="I83" s="24" t="s">
+        <v>251</v>
+      </c>
       <c r="J83" s="24" t="s">
-        <v>474</v>
+        <v>250</v>
       </c>
       <c r="Q83" s="24" t="s">
         <v>391</v>
@@ -8878,7 +8854,7 @@
     </row>
     <row r="84">
       <c r="A84" s="24" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B84" s="29">
         <v>46186.0</v>
@@ -8900,7 +8876,7 @@
         <v>17</v>
       </c>
       <c r="J84" s="24" t="s">
-        <v>476</v>
+        <v>252</v>
       </c>
       <c r="Q84" s="24" t="s">
         <v>391</v>
@@ -8908,7 +8884,7 @@
     </row>
     <row r="85">
       <c r="A85" s="24" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B85" s="29">
         <v>46186.0</v>
@@ -8929,8 +8905,11 @@
       <c r="H85" s="24" t="s">
         <v>17</v>
       </c>
+      <c r="I85" s="24" t="s">
+        <v>254</v>
+      </c>
       <c r="J85" s="24" t="s">
-        <v>478</v>
+        <v>253</v>
       </c>
       <c r="Q85" s="24" t="s">
         <v>391</v>
@@ -8938,7 +8917,7 @@
     </row>
     <row r="86">
       <c r="A86" s="24" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="B86" s="29">
         <v>46186.0</v>
@@ -8961,7 +8940,7 @@
       </c>
       <c r="I86" s="24"/>
       <c r="J86" s="24" t="s">
-        <v>480</v>
+        <v>257</v>
       </c>
       <c r="Q86" s="24" t="s">
         <v>391</v>
@@ -8969,7 +8948,7 @@
     </row>
     <row r="87">
       <c r="A87" s="24" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="B87" s="29">
         <v>46186.0</v>
@@ -8990,9 +8969,11 @@
       <c r="H87" s="24" t="s">
         <v>259</v>
       </c>
-      <c r="I87" s="24"/>
+      <c r="I87" s="25" t="s">
+        <v>261</v>
+      </c>
       <c r="J87" s="24" t="s">
-        <v>482</v>
+        <v>260</v>
       </c>
       <c r="Q87" s="24" t="s">
         <v>391</v>
@@ -9000,7 +8981,7 @@
     </row>
     <row r="88">
       <c r="A88" s="24" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="B88" s="29">
         <v>46186.0</v>
@@ -9023,7 +9004,7 @@
       </c>
       <c r="I88" s="24"/>
       <c r="J88" s="24" t="s">
-        <v>484</v>
+        <v>264</v>
       </c>
       <c r="Q88" s="24" t="s">
         <v>391</v>
@@ -9031,7 +9012,7 @@
     </row>
     <row r="89">
       <c r="A89" s="24" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="B89" s="29">
         <v>46186.0</v>
@@ -9054,7 +9035,7 @@
       </c>
       <c r="I89" s="24"/>
       <c r="J89" s="24" t="s">
-        <v>486</v>
+        <v>265</v>
       </c>
       <c r="Q89" s="24" t="s">
         <v>391</v>
@@ -9062,7 +9043,7 @@
     </row>
     <row r="90">
       <c r="A90" s="24" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="B90" s="29">
         <v>46186.0</v>
@@ -9083,9 +9064,11 @@
       <c r="H90" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I90" s="24"/>
+      <c r="I90" s="25" t="s">
+        <v>267</v>
+      </c>
       <c r="J90" s="24" t="s">
-        <v>488</v>
+        <v>266</v>
       </c>
       <c r="Q90" s="24" t="s">
         <v>391</v>
@@ -9093,7 +9076,7 @@
     </row>
     <row r="91">
       <c r="A91" s="24" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="B91" s="29">
         <v>46186.0</v>
@@ -9109,13 +9092,16 @@
         <v>258</v>
       </c>
       <c r="G91" s="24" t="s">
-        <v>14</v>
+        <v>268</v>
       </c>
       <c r="H91" s="24" t="s">
         <v>259</v>
       </c>
+      <c r="I91" s="24" t="s">
+        <v>270</v>
+      </c>
       <c r="J91" s="24" t="s">
-        <v>490</v>
+        <v>269</v>
       </c>
       <c r="Q91" s="24" t="s">
         <v>391</v>
@@ -9123,7 +9109,7 @@
     </row>
     <row r="92">
       <c r="A92" s="24" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
       <c r="B92" s="29">
         <v>46186.0</v>
@@ -9144,9 +9130,11 @@
       <c r="H92" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I92" s="24"/>
+      <c r="I92" s="25" t="s">
+        <v>273</v>
+      </c>
       <c r="J92" s="24" t="s">
-        <v>492</v>
+        <v>272</v>
       </c>
       <c r="Q92" s="24" t="s">
         <v>391</v>
@@ -9154,7 +9142,7 @@
     </row>
     <row r="93">
       <c r="A93" s="24" t="s">
-        <v>493</v>
+        <v>483</v>
       </c>
       <c r="B93" s="29">
         <v>46186.0</v>
@@ -9176,7 +9164,7 @@
         <v>259</v>
       </c>
       <c r="J93" s="24" t="s">
-        <v>494</v>
+        <v>274</v>
       </c>
       <c r="Q93" s="24" t="s">
         <v>391</v>
@@ -9184,7 +9172,7 @@
     </row>
     <row r="94">
       <c r="A94" s="24" t="s">
-        <v>495</v>
+        <v>484</v>
       </c>
       <c r="B94" s="29">
         <v>46186.0</v>
@@ -9205,8 +9193,11 @@
       <c r="H94" s="24" t="s">
         <v>17</v>
       </c>
+      <c r="I94" s="24" t="s">
+        <v>276</v>
+      </c>
       <c r="J94" s="24" t="s">
-        <v>496</v>
+        <v>275</v>
       </c>
       <c r="Q94" s="24" t="s">
         <v>391</v>
@@ -9214,7 +9205,7 @@
     </row>
     <row r="95">
       <c r="A95" s="24" t="s">
-        <v>497</v>
+        <v>485</v>
       </c>
       <c r="B95" s="29">
         <v>46186.0</v>
@@ -9235,8 +9226,11 @@
       <c r="H95" s="24" t="s">
         <v>17</v>
       </c>
+      <c r="I95" s="25" t="s">
+        <v>279</v>
+      </c>
       <c r="J95" s="24" t="s">
-        <v>498</v>
+        <v>278</v>
       </c>
       <c r="Q95" s="24" t="s">
         <v>391</v>
@@ -9244,7 +9238,7 @@
     </row>
     <row r="96">
       <c r="A96" s="24" t="s">
-        <v>499</v>
+        <v>486</v>
       </c>
       <c r="B96" s="29">
         <v>46186.0</v>
@@ -9267,7 +9261,7 @@
       </c>
       <c r="I96" s="24"/>
       <c r="J96" s="24" t="s">
-        <v>500</v>
+        <v>281</v>
       </c>
       <c r="Q96" s="24" t="s">
         <v>391</v>
@@ -9275,7 +9269,7 @@
     </row>
     <row r="97">
       <c r="A97" s="24" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B97" s="29">
         <v>46186.0</v>
@@ -9296,9 +9290,11 @@
       <c r="H97" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I97" s="24"/>
+      <c r="I97" s="24" t="s">
+        <v>283</v>
+      </c>
       <c r="J97" s="24" t="s">
-        <v>502</v>
+        <v>282</v>
       </c>
       <c r="Q97" s="24" t="s">
         <v>391</v>
@@ -9306,7 +9302,7 @@
     </row>
     <row r="98">
       <c r="A98" s="24" t="s">
-        <v>503</v>
+        <v>488</v>
       </c>
       <c r="B98" s="29">
         <v>46186.0</v>
@@ -9327,8 +9323,11 @@
       <c r="H98" s="24" t="s">
         <v>17</v>
       </c>
+      <c r="I98" s="24" t="s">
+        <v>489</v>
+      </c>
       <c r="J98" s="24" t="s">
-        <v>504</v>
+        <v>284</v>
       </c>
       <c r="Q98" s="24" t="s">
         <v>391</v>
@@ -9336,7 +9335,7 @@
     </row>
     <row r="99">
       <c r="A99" s="24" t="s">
-        <v>505</v>
+        <v>490</v>
       </c>
       <c r="B99" s="29">
         <v>46186.0</v>
@@ -9357,8 +9356,11 @@
       <c r="H99" s="24" t="s">
         <v>286</v>
       </c>
+      <c r="I99" s="25" t="s">
+        <v>288</v>
+      </c>
       <c r="J99" s="24" t="s">
-        <v>506</v>
+        <v>287</v>
       </c>
       <c r="Q99" s="24" t="s">
         <v>391</v>
@@ -9366,7 +9368,7 @@
     </row>
     <row r="100">
       <c r="A100" s="24" t="s">
-        <v>507</v>
+        <v>491</v>
       </c>
       <c r="B100" s="29">
         <v>46186.0</v>
@@ -9386,9 +9388,11 @@
       <c r="H100" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I100" s="24"/>
+      <c r="I100" s="25" t="s">
+        <v>290</v>
+      </c>
       <c r="J100" s="24" t="s">
-        <v>508</v>
+        <v>289</v>
       </c>
       <c r="Q100" s="24" t="s">
         <v>391</v>
@@ -9396,7 +9400,7 @@
     </row>
     <row r="101">
       <c r="A101" s="24" t="s">
-        <v>509</v>
+        <v>492</v>
       </c>
       <c r="B101" s="29">
         <v>46186.0</v>
@@ -9418,7 +9422,7 @@
       </c>
       <c r="I101" s="24"/>
       <c r="J101" s="24" t="s">
-        <v>510</v>
+        <v>291</v>
       </c>
       <c r="Q101" s="24" t="s">
         <v>391</v>
@@ -9426,7 +9430,7 @@
     </row>
     <row r="102">
       <c r="A102" s="24" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
       <c r="B102" s="29">
         <v>46186.0</v>
@@ -9446,9 +9450,11 @@
       <c r="H102" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I102" s="24"/>
+      <c r="I102" s="24" t="s">
+        <v>494</v>
+      </c>
       <c r="J102" s="24" t="s">
-        <v>512</v>
+        <v>292</v>
       </c>
       <c r="Q102" s="24" t="s">
         <v>391</v>
@@ -9456,7 +9462,7 @@
     </row>
     <row r="103">
       <c r="A103" s="24" t="s">
-        <v>513</v>
+        <v>495</v>
       </c>
       <c r="B103" s="29">
         <v>46186.0</v>
@@ -9478,7 +9484,7 @@
       </c>
       <c r="I103" s="24"/>
       <c r="J103" s="24" t="s">
-        <v>514</v>
+        <v>294</v>
       </c>
       <c r="Q103" s="24" t="s">
         <v>391</v>
@@ -9486,7 +9492,7 @@
     </row>
     <row r="104">
       <c r="A104" s="24" t="s">
-        <v>515</v>
+        <v>496</v>
       </c>
       <c r="B104" s="29">
         <v>46186.0</v>
@@ -9506,9 +9512,11 @@
       <c r="H104" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="I104" s="24"/>
+      <c r="I104" s="24" t="s">
+        <v>296</v>
+      </c>
       <c r="J104" s="24" t="s">
-        <v>516</v>
+        <v>295</v>
       </c>
       <c r="Q104" s="24" t="s">
         <v>391</v>
@@ -9516,7 +9524,7 @@
     </row>
     <row r="105">
       <c r="A105" s="24" t="s">
-        <v>517</v>
+        <v>497</v>
       </c>
       <c r="B105" s="29">
         <v>46186.0</v>
@@ -9536,8 +9544,11 @@
       <c r="H105" s="24" t="s">
         <v>286</v>
       </c>
+      <c r="I105" s="24" t="s">
+        <v>498</v>
+      </c>
       <c r="J105" s="24" t="s">
-        <v>518</v>
+        <v>298</v>
       </c>
       <c r="Q105" s="24" t="s">
         <v>391</v>
@@ -9545,7 +9556,7 @@
     </row>
     <row r="106">
       <c r="A106" s="24" t="s">
-        <v>519</v>
+        <v>499</v>
       </c>
       <c r="B106" s="29">
         <v>46186.0</v>
@@ -9567,7 +9578,7 @@
       </c>
       <c r="I106" s="24"/>
       <c r="J106" s="24" t="s">
-        <v>520</v>
+        <v>300</v>
       </c>
       <c r="Q106" s="24" t="s">
         <v>391</v>
@@ -9575,7 +9586,7 @@
     </row>
     <row r="107">
       <c r="A107" s="24" t="s">
-        <v>521</v>
+        <v>500</v>
       </c>
       <c r="B107" s="29">
         <v>46179.0</v>
@@ -9600,7 +9611,7 @@
     </row>
     <row r="108">
       <c r="A108" s="24" t="s">
-        <v>522</v>
+        <v>501</v>
       </c>
       <c r="B108" s="29">
         <v>46179.0</v>
@@ -9625,7 +9636,7 @@
     </row>
     <row r="109">
       <c r="A109" s="24" t="s">
-        <v>523</v>
+        <v>502</v>
       </c>
       <c r="B109" s="29">
         <v>46179.0</v>
@@ -9650,7 +9661,7 @@
     </row>
     <row r="110">
       <c r="A110" s="24" t="s">
-        <v>524</v>
+        <v>503</v>
       </c>
       <c r="B110" s="29">
         <v>46179.0</v>
@@ -9675,7 +9686,7 @@
     </row>
     <row r="111">
       <c r="A111" s="24" t="s">
-        <v>525</v>
+        <v>504</v>
       </c>
       <c r="B111" s="29">
         <v>46179.0</v>
@@ -9700,7 +9711,7 @@
     </row>
     <row r="112">
       <c r="A112" s="24" t="s">
-        <v>526</v>
+        <v>505</v>
       </c>
       <c r="B112" s="29">
         <v>46179.0</v>
@@ -9725,7 +9736,7 @@
     </row>
     <row r="113">
       <c r="A113" s="24" t="s">
-        <v>527</v>
+        <v>506</v>
       </c>
       <c r="B113" s="29">
         <v>46179.0</v>
@@ -9750,7 +9761,7 @@
     </row>
     <row r="114">
       <c r="A114" s="24" t="s">
-        <v>528</v>
+        <v>507</v>
       </c>
       <c r="B114" s="29">
         <v>46179.0</v>
@@ -9775,7 +9786,7 @@
     </row>
     <row r="115">
       <c r="A115" s="24" t="s">
-        <v>529</v>
+        <v>508</v>
       </c>
       <c r="B115" s="29">
         <v>46179.0</v>
@@ -9800,7 +9811,7 @@
     </row>
     <row r="116">
       <c r="A116" s="24" t="s">
-        <v>530</v>
+        <v>509</v>
       </c>
       <c r="B116" s="29">
         <v>46179.0</v>
@@ -9825,7 +9836,7 @@
     </row>
     <row r="117">
       <c r="A117" s="24" t="s">
-        <v>531</v>
+        <v>510</v>
       </c>
       <c r="B117" s="29">
         <v>46179.0</v>
@@ -9850,7 +9861,7 @@
     </row>
     <row r="118">
       <c r="A118" s="24" t="s">
-        <v>532</v>
+        <v>511</v>
       </c>
       <c r="B118" s="29">
         <v>46179.0</v>
@@ -9875,7 +9886,7 @@
     </row>
     <row r="119">
       <c r="A119" s="24" t="s">
-        <v>533</v>
+        <v>512</v>
       </c>
       <c r="B119" s="29">
         <v>46179.0</v>
@@ -9900,7 +9911,7 @@
     </row>
     <row r="120">
       <c r="A120" s="24" t="s">
-        <v>534</v>
+        <v>513</v>
       </c>
       <c r="B120" s="29">
         <v>46179.0</v>
@@ -9925,7 +9936,7 @@
     </row>
     <row r="121">
       <c r="A121" s="24" t="s">
-        <v>535</v>
+        <v>514</v>
       </c>
       <c r="B121" s="29">
         <v>46179.0</v>
@@ -9949,7 +9960,7 @@
     </row>
     <row r="122">
       <c r="A122" s="24" t="s">
-        <v>536</v>
+        <v>515</v>
       </c>
       <c r="B122" s="29">
         <v>46179.0</v>
@@ -9973,7 +9984,7 @@
     </row>
     <row r="123">
       <c r="A123" s="24" t="s">
-        <v>537</v>
+        <v>516</v>
       </c>
       <c r="B123" s="29">
         <v>46179.0</v>
@@ -9997,7 +10008,7 @@
     </row>
     <row r="124">
       <c r="A124" s="24" t="s">
-        <v>538</v>
+        <v>517</v>
       </c>
       <c r="B124" s="29">
         <v>46179.0</v>
@@ -10021,7 +10032,7 @@
     </row>
     <row r="125">
       <c r="A125" s="24" t="s">
-        <v>539</v>
+        <v>518</v>
       </c>
       <c r="B125" s="29">
         <v>46179.0</v>
@@ -10044,91 +10055,264 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="24"/>
-      <c r="B126" s="28"/>
-      <c r="C126" s="24"/>
-      <c r="E126" s="24"/>
-      <c r="F126" s="24"/>
-      <c r="H126" s="24"/>
-      <c r="J126" s="24"/>
-      <c r="Q126" s="24"/>
+      <c r="A126" s="24" t="s">
+        <v>519</v>
+      </c>
+      <c r="B126" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C126" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="E126" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F126" s="24" t="s">
+        <v>320</v>
+      </c>
+      <c r="G126" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H126" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I126" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="J126" s="24" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q126" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="24"/>
-      <c r="B127" s="28"/>
-      <c r="C127" s="24"/>
-      <c r="E127" s="24"/>
-      <c r="F127" s="24"/>
-      <c r="H127" s="24"/>
-      <c r="J127" s="24"/>
-      <c r="Q127" s="24"/>
+      <c r="A127" s="24" t="s">
+        <v>520</v>
+      </c>
+      <c r="B127" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C127" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="E127" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F127" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="G127" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H127" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I127" s="24" t="s">
+        <v>521</v>
+      </c>
+      <c r="J127" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q127" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="24"/>
-      <c r="B128" s="28"/>
-      <c r="C128" s="24"/>
-      <c r="E128" s="24"/>
-      <c r="F128" s="24"/>
-      <c r="H128" s="24"/>
-      <c r="J128" s="24"/>
-      <c r="Q128" s="24"/>
+      <c r="A128" s="24" t="s">
+        <v>522</v>
+      </c>
+      <c r="B128" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C128" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="E128" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F128" s="24" t="s">
+        <v>263</v>
+      </c>
+      <c r="G128" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H128" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I128" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="J128" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q128" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="24"/>
-      <c r="B129" s="28"/>
-      <c r="C129" s="24"/>
-      <c r="E129" s="24"/>
-      <c r="F129" s="24"/>
-      <c r="H129" s="24"/>
-      <c r="J129" s="24"/>
-      <c r="Q129" s="24"/>
+      <c r="A129" s="24" t="s">
+        <v>523</v>
+      </c>
+      <c r="B129" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C129" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="E129" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F129" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="G129" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H129" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I129" s="24" t="s">
+        <v>524</v>
+      </c>
+      <c r="J129" s="24" t="s">
+        <v>327</v>
+      </c>
+      <c r="Q129" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="24"/>
-      <c r="B130" s="28"/>
-      <c r="C130" s="24"/>
+      <c r="A130" s="24" t="s">
+        <v>525</v>
+      </c>
+      <c r="B130" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C130" s="24" t="s">
+        <v>248</v>
+      </c>
       <c r="D130" s="24"/>
-      <c r="E130" s="24"/>
-      <c r="F130" s="24"/>
-      <c r="H130" s="24"/>
-      <c r="I130" s="24"/>
-      <c r="J130" s="24"/>
-      <c r="Q130" s="24"/>
+      <c r="E130" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F130" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G130" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H130" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I130" s="24" t="s">
+        <v>526</v>
+      </c>
+      <c r="J130" s="24" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q130" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="24"/>
-      <c r="B131" s="28"/>
-      <c r="C131" s="24"/>
+      <c r="A131" s="24" t="s">
+        <v>527</v>
+      </c>
+      <c r="B131" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C131" s="24" t="s">
+        <v>248</v>
+      </c>
       <c r="D131" s="24"/>
-      <c r="E131" s="24"/>
-      <c r="F131" s="24"/>
-      <c r="H131" s="24"/>
-      <c r="I131" s="24"/>
-      <c r="J131" s="24"/>
-      <c r="Q131" s="24"/>
+      <c r="E131" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F131" s="24" t="s">
+        <v>331</v>
+      </c>
+      <c r="G131" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="H131" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I131" s="24" t="s">
+        <v>528</v>
+      </c>
+      <c r="J131" s="24" t="s">
+        <v>332</v>
+      </c>
+      <c r="Q131" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="24"/>
-      <c r="B132" s="28"/>
-      <c r="C132" s="24"/>
+      <c r="A132" s="24" t="s">
+        <v>529</v>
+      </c>
+      <c r="B132" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C132" s="24" t="s">
+        <v>248</v>
+      </c>
       <c r="D132" s="24"/>
-      <c r="E132" s="24"/>
-      <c r="F132" s="24"/>
-      <c r="H132" s="24"/>
-      <c r="J132" s="24"/>
-      <c r="Q132" s="24"/>
+      <c r="E132" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F132" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G132" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H132" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I132" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="J132" s="24" t="s">
+        <v>334</v>
+      </c>
+      <c r="Q132" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="24"/>
-      <c r="B133" s="28"/>
-      <c r="C133" s="24"/>
+      <c r="A133" s="24" t="s">
+        <v>530</v>
+      </c>
+      <c r="B133" s="29">
+        <v>46186.0</v>
+      </c>
+      <c r="C133" s="24" t="s">
+        <v>248</v>
+      </c>
       <c r="D133" s="24"/>
-      <c r="E133" s="24"/>
-      <c r="F133" s="24"/>
-      <c r="H133" s="24"/>
-      <c r="I133" s="24"/>
-      <c r="J133" s="24"/>
-      <c r="Q133" s="24"/>
+      <c r="E133" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="F133" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G133" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H133" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="I133" s="25" t="s">
+        <v>337</v>
+      </c>
+      <c r="J133" s="24" t="s">
+        <v>336</v>
+      </c>
+      <c r="Q133" s="24" t="s">
+        <v>391</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="24"/>
@@ -10431,8 +10615,17 @@
     <hyperlink r:id="rId27" ref="I78"/>
     <hyperlink r:id="rId28" ref="I79"/>
     <hyperlink r:id="rId29" ref="I82"/>
+    <hyperlink r:id="rId30" ref="I87"/>
+    <hyperlink r:id="rId31" ref="I90"/>
+    <hyperlink r:id="rId32" ref="I92"/>
+    <hyperlink r:id="rId33" ref="I95"/>
+    <hyperlink r:id="rId34" ref="I99"/>
+    <hyperlink r:id="rId35" ref="I100"/>
+    <hyperlink r:id="rId36" ref="I126"/>
+    <hyperlink r:id="rId37" ref="I132"/>
+    <hyperlink r:id="rId38" ref="I133"/>
   </hyperlinks>
-  <drawing r:id="rId30"/>
+  <drawing r:id="rId39"/>
 </worksheet>
 </file>
 
@@ -10468,64 +10661,64 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="32" t="s">
-        <v>540</v>
+        <v>531</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>541</v>
+        <v>532</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>542</v>
+        <v>533</v>
       </c>
       <c r="D1" s="32" t="s">
-        <v>543</v>
+        <v>534</v>
       </c>
       <c r="E1" s="32" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="32" t="s">
-        <v>544</v>
+        <v>535</v>
       </c>
       <c r="G1" s="32" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="32" t="s">
-        <v>545</v>
+        <v>536</v>
       </c>
       <c r="I1" s="32" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="32" t="s">
+        <v>537</v>
+      </c>
+      <c r="K1" s="32" t="s">
+        <v>538</v>
+      </c>
+      <c r="L1" s="32" t="s">
+        <v>539</v>
+      </c>
+      <c r="M1" s="32" t="s">
+        <v>540</v>
+      </c>
+      <c r="N1" s="32" t="s">
+        <v>541</v>
+      </c>
+      <c r="O1" s="32" t="s">
+        <v>542</v>
+      </c>
+      <c r="P1" s="32" t="s">
+        <v>543</v>
+      </c>
+      <c r="Q1" s="32" t="s">
+        <v>544</v>
+      </c>
+      <c r="R1" s="32" t="s">
+        <v>545</v>
+      </c>
+      <c r="S1" s="32" t="s">
         <v>546</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="T1" s="32" t="s">
         <v>547</v>
-      </c>
-      <c r="L1" s="32" t="s">
-        <v>548</v>
-      </c>
-      <c r="M1" s="32" t="s">
-        <v>549</v>
-      </c>
-      <c r="N1" s="32" t="s">
-        <v>550</v>
-      </c>
-      <c r="O1" s="32" t="s">
-        <v>551</v>
-      </c>
-      <c r="P1" s="32" t="s">
-        <v>552</v>
-      </c>
-      <c r="Q1" s="32" t="s">
-        <v>553</v>
-      </c>
-      <c r="R1" s="32" t="s">
-        <v>554</v>
-      </c>
-      <c r="S1" s="32" t="s">
-        <v>555</v>
-      </c>
-      <c r="T1" s="32" t="s">
-        <v>556</v>
       </c>
     </row>
     <row r="2">
@@ -18723,7 +18916,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>545</v>
+        <v>536</v>
       </c>
       <c r="C1" s="32" t="s">
         <v>5</v>
@@ -18732,7 +18925,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="32" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
     </row>
     <row r="2">
@@ -18749,7 +18942,7 @@
         <v>35</v>
       </c>
       <c r="E2" s="34" t="s">
-        <v>557</v>
+        <v>548</v>
       </c>
     </row>
     <row r="3">
@@ -18766,7 +18959,7 @@
         <v>15</v>
       </c>
       <c r="E3" s="34" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
     </row>
     <row r="4">
@@ -18783,7 +18976,7 @@
         <v>45</v>
       </c>
       <c r="E4" s="34" t="s">
-        <v>559</v>
+        <v>550</v>
       </c>
     </row>
     <row r="5">
@@ -18800,7 +18993,7 @@
         <v>17</v>
       </c>
       <c r="E5" s="34" t="s">
-        <v>560</v>
+        <v>551</v>
       </c>
     </row>
     <row r="6">
@@ -18832,12 +19025,12 @@
         <v>17</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>561</v>
+        <v>552</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="34" t="s">
-        <v>562</v>
+        <v>553</v>
       </c>
       <c r="B10" s="34" t="s">
         <v>133</v>
@@ -18850,7 +19043,7 @@
     </row>
     <row r="12">
       <c r="B12" s="34" t="s">
-        <v>563</v>
+        <v>554</v>
       </c>
     </row>
     <row r="13">
@@ -18860,7 +19053,7 @@
     </row>
     <row r="14">
       <c r="B14" s="34" t="s">
-        <v>564</v>
+        <v>555</v>
       </c>
     </row>
     <row r="15">
@@ -18870,7 +19063,7 @@
     </row>
     <row r="16">
       <c r="B16" s="34" t="s">
-        <v>565</v>
+        <v>556</v>
       </c>
     </row>
     <row r="17">
@@ -18880,12 +19073,12 @@
     </row>
     <row r="18">
       <c r="B18" s="34" t="s">
-        <v>566</v>
+        <v>557</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="34" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
     </row>
     <row r="20">
@@ -18900,7 +19093,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="34" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -18910,7 +19103,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="34" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1"/>

</xml_diff>